<commit_message>
Update data tgl 31 Agustus, sync Supabase, bump cache version v3.3, and update agent skill
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -18,6 +18,7 @@
     <sheet name="28 Agustus" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="29 Agustus" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="30 Agustus" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="31 Agustus" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;kg&quot;"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,8 +96,28 @@
       <color rgb="00475569"/>
       <sz val="9.5"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -151,8 +172,14 @@
         <bgColor rgb="00334155"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -188,11 +215,89 @@
         <color rgb="001D1D1B"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001D1D1B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="medium">
+        <color rgb="001D1D1B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001D1D1B"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001D1D1B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="medium">
+        <color rgb="001D1D1B"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001D1D1B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color rgb="001D1D1B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -283,6 +388,28 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -650,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H463"/>
+  <dimension ref="A1:H482"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -673,11 +800,10 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Laporan Lengkap No Gudang, Nomor Barcode, Grade, dan Berat (Kg) Semua Tanggal (21 - 30 Agustus 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Laporan Lengkap No Gudang, Nomor Barcode, Grade, dan Berat (Kg) Semua Tanggal (21 - 31 Agustus 2026)</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -17111,27 +17237,712 @@
       </c>
     </row>
     <row r="463" ht="24" customHeight="1">
-      <c r="A463" s="20" t="inlineStr">
+      <c r="A463" s="32" t="n">
+        <v>459</v>
+      </c>
+      <c r="B463" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C463" s="32" t="n">
+        <v>605</v>
+      </c>
+      <c r="D463" s="33" t="inlineStr">
+        <is>
+          <t>34953</t>
+        </is>
+      </c>
+      <c r="E463" s="32" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F463" s="32" t="n">
+        <v>38</v>
+      </c>
+      <c r="G463" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H463" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="32" t="n">
+        <v>460</v>
+      </c>
+      <c r="B464" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C464" s="32" t="n">
+        <v>607</v>
+      </c>
+      <c r="D464" s="33" t="inlineStr">
+        <is>
+          <t>33854</t>
+        </is>
+      </c>
+      <c r="E464" s="32" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F464" s="32" t="n">
+        <v>35</v>
+      </c>
+      <c r="G464" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H464" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="32" t="n">
+        <v>461</v>
+      </c>
+      <c r="B465" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C465" s="32" t="n">
+        <v>608</v>
+      </c>
+      <c r="D465" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E465" s="32" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F465" s="32" t="n">
+        <v>42</v>
+      </c>
+      <c r="G465" s="32" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="H465" s="34" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="32" t="n">
+        <v>462</v>
+      </c>
+      <c r="B466" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C466" s="32" t="n">
+        <v>609</v>
+      </c>
+      <c r="D466" s="33" t="inlineStr">
+        <is>
+          <t>34956</t>
+        </is>
+      </c>
+      <c r="E466" s="32" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="F466" s="32" t="n">
+        <v>31</v>
+      </c>
+      <c r="G466" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H466" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="32" t="n">
+        <v>463</v>
+      </c>
+      <c r="B467" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C467" s="32" t="n">
+        <v>610</v>
+      </c>
+      <c r="D467" s="33" t="inlineStr">
+        <is>
+          <t>35004</t>
+        </is>
+      </c>
+      <c r="E467" s="32" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="F467" s="32" t="n">
+        <v>41</v>
+      </c>
+      <c r="G467" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H467" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="32" t="n">
+        <v>464</v>
+      </c>
+      <c r="B468" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C468" s="32" t="n">
+        <v>611</v>
+      </c>
+      <c r="D468" s="33" t="inlineStr">
+        <is>
+          <t>34394</t>
+        </is>
+      </c>
+      <c r="E468" s="32" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F468" s="32" t="n">
+        <v>35</v>
+      </c>
+      <c r="G468" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H468" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="32" t="n">
+        <v>465</v>
+      </c>
+      <c r="B469" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C469" s="32" t="n">
+        <v>612</v>
+      </c>
+      <c r="D469" s="33" t="inlineStr">
+        <is>
+          <t>35003</t>
+        </is>
+      </c>
+      <c r="E469" s="32" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F469" s="32" t="n">
+        <v>42</v>
+      </c>
+      <c r="G469" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H469" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="32" t="n">
+        <v>466</v>
+      </c>
+      <c r="B470" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C470" s="32" t="n">
+        <v>613</v>
+      </c>
+      <c r="D470" s="33" t="inlineStr">
+        <is>
+          <t>34954</t>
+        </is>
+      </c>
+      <c r="E470" s="32" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F470" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="G470" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H470" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="32" t="n">
+        <v>467</v>
+      </c>
+      <c r="B471" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C471" s="32" t="n">
+        <v>614</v>
+      </c>
+      <c r="D471" s="33" t="inlineStr">
+        <is>
+          <t>35002</t>
+        </is>
+      </c>
+      <c r="E471" s="32" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F471" s="32" t="n">
+        <v>31</v>
+      </c>
+      <c r="G471" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H471" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="32" t="n">
+        <v>468</v>
+      </c>
+      <c r="B472" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C472" s="32" t="n">
+        <v>615</v>
+      </c>
+      <c r="D472" s="33" t="inlineStr">
+        <is>
+          <t>35711</t>
+        </is>
+      </c>
+      <c r="E472" s="32" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F472" s="32" t="n">
+        <v>34</v>
+      </c>
+      <c r="G472" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H472" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="32" t="n">
+        <v>469</v>
+      </c>
+      <c r="B473" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C473" s="32" t="n">
+        <v>616</v>
+      </c>
+      <c r="D473" s="33" t="inlineStr">
+        <is>
+          <t>34955</t>
+        </is>
+      </c>
+      <c r="E473" s="32" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F473" s="32" t="n">
+        <v>39</v>
+      </c>
+      <c r="G473" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H473" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="32" t="n">
+        <v>470</v>
+      </c>
+      <c r="B474" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C474" s="32" t="n">
+        <v>618</v>
+      </c>
+      <c r="D474" s="33" t="inlineStr">
+        <is>
+          <t>34899</t>
+        </is>
+      </c>
+      <c r="E474" s="32" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F474" s="32" t="n">
+        <v>45</v>
+      </c>
+      <c r="G474" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H474" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="32" t="n">
+        <v>471</v>
+      </c>
+      <c r="B475" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C475" s="32" t="n">
+        <v>617</v>
+      </c>
+      <c r="D475" s="33" t="inlineStr">
+        <is>
+          <t>34285</t>
+        </is>
+      </c>
+      <c r="E475" s="32" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F475" s="32" t="n">
+        <v>36</v>
+      </c>
+      <c r="G475" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H475" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="32" t="n">
+        <v>472</v>
+      </c>
+      <c r="B476" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C476" s="32" t="n">
+        <v>619</v>
+      </c>
+      <c r="D476" s="33" t="inlineStr">
+        <is>
+          <t>35001</t>
+        </is>
+      </c>
+      <c r="E476" s="32" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F476" s="32" t="n">
+        <v>36</v>
+      </c>
+      <c r="G476" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H476" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="32" t="n">
+        <v>473</v>
+      </c>
+      <c r="B477" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C477" s="32" t="n">
+        <v>624</v>
+      </c>
+      <c r="D477" s="33" t="inlineStr">
+        <is>
+          <t>34393</t>
+        </is>
+      </c>
+      <c r="E477" s="32" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F477" s="32" t="n">
+        <v>34</v>
+      </c>
+      <c r="G477" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H477" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="32" t="n">
+        <v>474</v>
+      </c>
+      <c r="B478" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C478" s="32" t="n">
+        <v>621</v>
+      </c>
+      <c r="D478" s="33" t="inlineStr">
+        <is>
+          <t>34952</t>
+        </is>
+      </c>
+      <c r="E478" s="32" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F478" s="32" t="n">
+        <v>42</v>
+      </c>
+      <c r="G478" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H478" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="32" t="n">
+        <v>475</v>
+      </c>
+      <c r="B479" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C479" s="32" t="n">
+        <v>620</v>
+      </c>
+      <c r="D479" s="33" t="inlineStr">
+        <is>
+          <t>34951</t>
+        </is>
+      </c>
+      <c r="E479" s="32" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F479" s="32" t="n">
+        <v>31</v>
+      </c>
+      <c r="G479" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H479" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="32" t="n">
+        <v>476</v>
+      </c>
+      <c r="B480" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C480" s="32" t="n">
+        <v>622</v>
+      </c>
+      <c r="D480" s="33" t="inlineStr">
+        <is>
+          <t>34900</t>
+        </is>
+      </c>
+      <c r="E480" s="32" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F480" s="32" t="n">
+        <v>39</v>
+      </c>
+      <c r="G480" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H480" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="32" t="n">
+        <v>477</v>
+      </c>
+      <c r="B481" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C481" s="32" t="n">
+        <v>623</v>
+      </c>
+      <c r="D481" s="33" t="inlineStr">
+        <is>
+          <t>31988</t>
+        </is>
+      </c>
+      <c r="E481" s="32" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F481" s="32" t="n">
+        <v>38</v>
+      </c>
+      <c r="G481" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H481" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="35" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B463" s="21" t="n"/>
-      <c r="C463" s="21" t="n"/>
-      <c r="D463" s="21" t="n"/>
-      <c r="E463" s="21" t="n"/>
-      <c r="F463" s="22">
-        <f>SUM(F5:F462)</f>
+      <c r="B482" s="36" t="n"/>
+      <c r="C482" s="36" t="n"/>
+      <c r="D482" s="36" t="n"/>
+      <c r="E482" s="36" t="n"/>
+      <c r="F482" s="35">
+        <f>SUM(F5:F481)</f>
         <v/>
       </c>
-      <c r="G463" s="23">
-        <f>COUNTA(A5:A462) &amp; " Bal"</f>
+      <c r="G482" s="35">
+        <f>COUNTA(A5:A481) &amp; " Bal"</f>
         <v/>
       </c>
-      <c r="H463" s="21" t="inlineStr"/>
+      <c r="H482" s="37" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A482:E482"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A463:E463"/>
     <mergeCell ref="A1:H1"/>
@@ -17172,7 +17983,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -18828,9 +19638,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B57" s="21" t="n"/>
-      <c r="C57" s="21" t="n"/>
-      <c r="D57" s="21" t="n"/>
+      <c r="B57" s="38" t="n"/>
+      <c r="C57" s="38" t="n"/>
+      <c r="D57" s="39" t="n"/>
       <c r="E57" s="22">
         <f>SUM(E5:E56)</f>
         <v/>
@@ -18883,7 +19693,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -19574,9 +20383,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B26" s="21" t="n"/>
-      <c r="C26" s="21" t="n"/>
-      <c r="D26" s="21" t="n"/>
+      <c r="B26" s="38" t="n"/>
+      <c r="C26" s="38" t="n"/>
+      <c r="D26" s="39" t="n"/>
       <c r="E26" s="22">
         <f>SUM(E5:E25)</f>
         <v/>
@@ -19592,6 +20401,690 @@
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="40" t="inlineStr">
+        <is>
+          <t>T.B.K JH — REKAPITULASI HARIAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="41" t="inlineStr">
+        <is>
+          <t>Data Bal Gudang Induk Tanggal: 31 Agustus 2026 (Senin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>No Gud</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>Nomor Barkot</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="35" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="32" t="n">
+        <v>605</v>
+      </c>
+      <c r="C5" s="33" t="inlineStr">
+        <is>
+          <t>34953</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E5" s="32" t="n">
+        <v>38</v>
+      </c>
+      <c r="F5" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="32" t="n">
+        <v>607</v>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>33854</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E6" s="32" t="n">
+        <v>35</v>
+      </c>
+      <c r="F6" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="32" t="n">
+        <v>608</v>
+      </c>
+      <c r="C7" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="n">
+        <v>42</v>
+      </c>
+      <c r="F7" s="32" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G7" s="34" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="32" t="n">
+        <v>609</v>
+      </c>
+      <c r="C8" s="33" t="inlineStr">
+        <is>
+          <t>34956</t>
+        </is>
+      </c>
+      <c r="D8" s="32" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E8" s="32" t="n">
+        <v>31</v>
+      </c>
+      <c r="F8" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="32" t="n">
+        <v>610</v>
+      </c>
+      <c r="C9" s="33" t="inlineStr">
+        <is>
+          <t>35004</t>
+        </is>
+      </c>
+      <c r="D9" s="32" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="E9" s="32" t="n">
+        <v>41</v>
+      </c>
+      <c r="F9" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="32" t="n">
+        <v>611</v>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>34394</t>
+        </is>
+      </c>
+      <c r="D10" s="32" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E10" s="32" t="n">
+        <v>35</v>
+      </c>
+      <c r="F10" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="32" t="n">
+        <v>612</v>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>35003</t>
+        </is>
+      </c>
+      <c r="D11" s="32" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="n">
+        <v>42</v>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="32" t="n">
+        <v>613</v>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>34954</t>
+        </is>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E12" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="32" t="n">
+        <v>614</v>
+      </c>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>35002</t>
+        </is>
+      </c>
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E13" s="32" t="n">
+        <v>31</v>
+      </c>
+      <c r="F13" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="32" t="n">
+        <v>615</v>
+      </c>
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>35711</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E14" s="32" t="n">
+        <v>34</v>
+      </c>
+      <c r="F14" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="32" t="n">
+        <v>616</v>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>34955</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="n">
+        <v>39</v>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="32" t="n">
+        <v>618</v>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>34899</t>
+        </is>
+      </c>
+      <c r="D16" s="32" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E16" s="32" t="n">
+        <v>45</v>
+      </c>
+      <c r="F16" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="32" t="n">
+        <v>617</v>
+      </c>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>34285</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E17" s="32" t="n">
+        <v>36</v>
+      </c>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="32" t="n">
+        <v>619</v>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>35001</t>
+        </is>
+      </c>
+      <c r="D18" s="32" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E18" s="32" t="n">
+        <v>36</v>
+      </c>
+      <c r="F18" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="32" t="n">
+        <v>624</v>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>34393</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E19" s="32" t="n">
+        <v>34</v>
+      </c>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="32" t="n">
+        <v>621</v>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>34952</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E20" s="32" t="n">
+        <v>42</v>
+      </c>
+      <c r="F20" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="32" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="32" t="n">
+        <v>620</v>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
+        <is>
+          <t>34951</t>
+        </is>
+      </c>
+      <c r="D21" s="32" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E21" s="32" t="n">
+        <v>31</v>
+      </c>
+      <c r="F21" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="32" t="n">
+        <v>622</v>
+      </c>
+      <c r="C22" s="33" t="inlineStr">
+        <is>
+          <t>34900</t>
+        </is>
+      </c>
+      <c r="D22" s="32" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E22" s="32" t="n">
+        <v>39</v>
+      </c>
+      <c r="F22" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="32" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="32" t="n">
+        <v>623</v>
+      </c>
+      <c r="C23" s="33" t="inlineStr">
+        <is>
+          <t>31988</t>
+        </is>
+      </c>
+      <c r="D23" s="32" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E23" s="32" t="n">
+        <v>38</v>
+      </c>
+      <c r="F23" s="32" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL (19 BAL)</t>
+        </is>
+      </c>
+      <c r="B24" s="36" t="n"/>
+      <c r="C24" s="36" t="n"/>
+      <c r="D24" s="36" t="n"/>
+      <c r="E24" s="35">
+        <f>SUM(E5:E23)</f>
+        <v/>
+      </c>
+      <c r="F24" s="37" t="n"/>
+      <c r="G24" s="37" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A24:D24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19603,7 +21096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19629,7 +21122,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -19893,35 +21385,61 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B14" s="21" t="n"/>
-      <c r="C14" s="23">
-        <f>SUM(C5:C13)</f>
+      <c r="A14" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>Senin</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="n">
+        <v>19</v>
+      </c>
+      <c r="E14" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="F14" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="32">
+        <f>SUM('31 Agustus'!E5:E23)</f>
         <v/>
       </c>
-      <c r="D14" s="23">
-        <f>SUM(D5:D13)</f>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL KESELURUHAN</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="n"/>
+      <c r="C15" s="36" t="n"/>
+      <c r="D15" s="35">
+        <f>SUM(D5:D14)</f>
         <v/>
       </c>
-      <c r="E14" s="23">
-        <f>SUM(E5:E13)</f>
+      <c r="E15" s="35">
+        <f>SUM(E5:E14)</f>
         <v/>
       </c>
-      <c r="F14" s="23">
-        <f>SUM(F5:F13)</f>
+      <c r="F15" s="35">
+        <f>SUM(F5:F14)</f>
         <v/>
       </c>
-      <c r="G14" s="22">
-        <f>SUM(G5:G13)</f>
+      <c r="G15" s="35">
+        <f>SUM(G5:G14)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
@@ -19962,7 +21480,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -21891,9 +23408,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B66" s="21" t="n"/>
-      <c r="C66" s="21" t="n"/>
-      <c r="D66" s="21" t="n"/>
+      <c r="B66" s="38" t="n"/>
+      <c r="C66" s="38" t="n"/>
+      <c r="D66" s="39" t="n"/>
       <c r="E66" s="22">
         <f>SUM(E5:E65)</f>
         <v/>
@@ -21946,7 +23463,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -23875,9 +25391,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B66" s="21" t="n"/>
-      <c r="C66" s="21" t="n"/>
-      <c r="D66" s="21" t="n"/>
+      <c r="B66" s="38" t="n"/>
+      <c r="C66" s="38" t="n"/>
+      <c r="D66" s="39" t="n"/>
       <c r="E66" s="22">
         <f>SUM(E5:E65)</f>
         <v/>
@@ -23930,7 +25446,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -25756,9 +27271,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B63" s="21" t="n"/>
-      <c r="C63" s="21" t="n"/>
-      <c r="D63" s="21" t="n"/>
+      <c r="B63" s="38" t="n"/>
+      <c r="C63" s="38" t="n"/>
+      <c r="D63" s="39" t="n"/>
       <c r="E63" s="22">
         <f>SUM(E5:E62)</f>
         <v/>
@@ -25811,7 +27326,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -27303,9 +28817,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B53" s="21" t="n"/>
-      <c r="C53" s="21" t="n"/>
-      <c r="D53" s="21" t="n"/>
+      <c r="B53" s="38" t="n"/>
+      <c r="C53" s="38" t="n"/>
+      <c r="D53" s="39" t="n"/>
       <c r="E53" s="22">
         <f>SUM(E5:E52)</f>
         <v/>
@@ -27358,7 +28872,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -29393,9 +30906,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B70" s="21" t="n"/>
-      <c r="C70" s="21" t="n"/>
-      <c r="D70" s="21" t="n"/>
+      <c r="B70" s="38" t="n"/>
+      <c r="C70" s="38" t="n"/>
+      <c r="D70" s="39" t="n"/>
       <c r="E70" s="22">
         <f>SUM(E5:E69)</f>
         <v/>
@@ -29448,7 +30961,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -31257,9 +32769,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B62" s="21" t="n"/>
-      <c r="C62" s="21" t="n"/>
-      <c r="D62" s="21" t="n"/>
+      <c r="B62" s="38" t="n"/>
+      <c r="C62" s="38" t="n"/>
+      <c r="D62" s="39" t="n"/>
       <c r="E62" s="22">
         <f>SUM(E5:E61)</f>
         <v/>
@@ -31312,7 +32824,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -32441,9 +33952,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B40" s="21" t="n"/>
-      <c r="C40" s="21" t="n"/>
-      <c r="D40" s="21" t="n"/>
+      <c r="B40" s="38" t="n"/>
+      <c r="C40" s="38" t="n"/>
+      <c r="D40" s="39" t="n"/>
       <c r="E40" s="22">
         <f>SUM(E5:E39)</f>
         <v/>

</xml_diff>

<commit_message>
Update data 1 September 2026, sync Supabase, and bump cache version v3.7
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -19,6 +19,7 @@
     <sheet name="29 Agustus" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="30 Agustus" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="31 Agustus" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="1 September" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +31,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;kg&quot;"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,6 +117,23 @@
       <i val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -179,7 +197,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -293,11 +311,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -411,6 +473,23 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -777,7 +856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H482"/>
+  <dimension ref="A1:H523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -800,7 +879,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Laporan Lengkap No Gudang, Nomor Barcode, Grade, dan Berat (Kg) Semua Tanggal (21 - 31 Agustus 2026)</t>
+          <t>Laporan Lengkap No Gudang, Nomor Barcode, Grade, dan Berat (Kg) Semua Tanggal (21 Agustus - 1 September 2026)</t>
         </is>
       </c>
     </row>
@@ -17240,24 +17319,10 @@
       <c r="A463" s="32" t="n">
         <v>459</v>
       </c>
-      <c r="B463" s="32" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C463" s="32" t="n">
-        <v>605</v>
-      </c>
-      <c r="D463" s="33" t="inlineStr">
-        <is>
-          <t>34953</t>
-        </is>
-      </c>
-      <c r="E463" s="32" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
+      <c r="B463" s="42" t="n"/>
+      <c r="C463" s="42" t="n"/>
+      <c r="D463" s="42" t="n"/>
+      <c r="E463" s="43" t="n"/>
       <c r="F463" s="32" t="n">
         <v>38</v>
       </c>
@@ -17920,32 +17985,1509 @@
         </is>
       </c>
     </row>
-    <row r="482">
-      <c r="A482" s="35" t="inlineStr">
-        <is>
-          <t>TOTAL KESELURUHAN</t>
-        </is>
-      </c>
-      <c r="B482" s="36" t="n"/>
-      <c r="C482" s="36" t="n"/>
-      <c r="D482" s="36" t="n"/>
-      <c r="E482" s="36" t="n"/>
-      <c r="F482" s="35">
-        <f>SUM(F5:F481)</f>
+    <row r="482" ht="20" customHeight="1">
+      <c r="A482" s="44" t="n">
+        <v>478</v>
+      </c>
+      <c r="B482" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C482" s="45" t="n">
+        <v>649</v>
+      </c>
+      <c r="D482" s="46" t="inlineStr">
+        <is>
+          <t>33863</t>
+        </is>
+      </c>
+      <c r="E482" s="45" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F482" s="44" t="n">
+        <v>38</v>
+      </c>
+      <c r="G482" s="44" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H482" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="483" ht="20" customHeight="1">
+      <c r="A483" s="45" t="n">
+        <v>479</v>
+      </c>
+      <c r="B483" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C483" s="45" t="n">
+        <v>647</v>
+      </c>
+      <c r="D483" s="46" t="inlineStr">
+        <is>
+          <t>33862</t>
+        </is>
+      </c>
+      <c r="E483" s="45" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F483" s="45" t="n">
+        <v>39</v>
+      </c>
+      <c r="G483" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H483" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="484" ht="20" customHeight="1">
+      <c r="A484" s="45" t="n">
+        <v>480</v>
+      </c>
+      <c r="B484" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C484" s="45" t="n">
+        <v>648</v>
+      </c>
+      <c r="D484" s="46" t="inlineStr">
+        <is>
+          <t>33861</t>
+        </is>
+      </c>
+      <c r="E484" s="45" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F484" s="45" t="n">
+        <v>40</v>
+      </c>
+      <c r="G484" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H484" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="485" ht="20" customHeight="1">
+      <c r="A485" s="45" t="n">
+        <v>481</v>
+      </c>
+      <c r="B485" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C485" s="45" t="n">
+        <v>644</v>
+      </c>
+      <c r="D485" s="46" t="inlineStr">
+        <is>
+          <t>35733</t>
+        </is>
+      </c>
+      <c r="E485" s="45" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F485" s="45" t="n">
+        <v>47</v>
+      </c>
+      <c r="G485" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H485" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="486" ht="20" customHeight="1">
+      <c r="A486" s="45" t="n">
+        <v>482</v>
+      </c>
+      <c r="B486" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C486" s="45" t="n">
+        <v>646</v>
+      </c>
+      <c r="D486" s="46" t="inlineStr">
+        <is>
+          <t>33860</t>
+        </is>
+      </c>
+      <c r="E486" s="45" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F486" s="45" t="n">
+        <v>42</v>
+      </c>
+      <c r="G486" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H486" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="487" ht="20" customHeight="1">
+      <c r="A487" s="45" t="n">
+        <v>483</v>
+      </c>
+      <c r="B487" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C487" s="45" t="n">
+        <v>645</v>
+      </c>
+      <c r="D487" s="46" t="inlineStr">
+        <is>
+          <t>35735</t>
+        </is>
+      </c>
+      <c r="E487" s="45" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="F487" s="45" t="n">
+        <v>43</v>
+      </c>
+      <c r="G487" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H487" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="488" ht="20" customHeight="1">
+      <c r="A488" s="45" t="n">
+        <v>484</v>
+      </c>
+      <c r="B488" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C488" s="45" t="n">
+        <v>643</v>
+      </c>
+      <c r="D488" s="46" t="inlineStr">
+        <is>
+          <t>35736</t>
+        </is>
+      </c>
+      <c r="E488" s="45" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="F488" s="45" t="n">
+        <v>46</v>
+      </c>
+      <c r="G488" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H488" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="489" ht="20" customHeight="1">
+      <c r="A489" s="45" t="n">
+        <v>485</v>
+      </c>
+      <c r="B489" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C489" s="45" t="n">
+        <v>637</v>
+      </c>
+      <c r="D489" s="46" t="inlineStr">
+        <is>
+          <t>35729</t>
+        </is>
+      </c>
+      <c r="E489" s="45" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="F489" s="45" t="n">
+        <v>49</v>
+      </c>
+      <c r="G489" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H489" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="490" ht="20" customHeight="1">
+      <c r="A490" s="45" t="n">
+        <v>486</v>
+      </c>
+      <c r="B490" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C490" s="45" t="n">
+        <v>639</v>
+      </c>
+      <c r="D490" s="46" t="inlineStr">
+        <is>
+          <t>35731</t>
+        </is>
+      </c>
+      <c r="E490" s="45" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="F490" s="45" t="n">
+        <v>41</v>
+      </c>
+      <c r="G490" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H490" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="491" ht="20" customHeight="1">
+      <c r="A491" s="45" t="n">
+        <v>487</v>
+      </c>
+      <c r="B491" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C491" s="45" t="n">
+        <v>650</v>
+      </c>
+      <c r="D491" s="46" t="inlineStr">
+        <is>
+          <t>35739</t>
+        </is>
+      </c>
+      <c r="E491" s="45" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F491" s="45" t="n">
+        <v>30</v>
+      </c>
+      <c r="G491" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H491" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="492" ht="20" customHeight="1">
+      <c r="A492" s="45" t="n">
+        <v>488</v>
+      </c>
+      <c r="B492" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C492" s="45" t="n">
+        <v>651</v>
+      </c>
+      <c r="D492" s="46" t="inlineStr">
+        <is>
+          <t>35738</t>
+        </is>
+      </c>
+      <c r="E492" s="45" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F492" s="45" t="n">
+        <v>41</v>
+      </c>
+      <c r="G492" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H492" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="493" ht="20" customHeight="1">
+      <c r="A493" s="45" t="n">
+        <v>489</v>
+      </c>
+      <c r="B493" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C493" s="45" t="n">
+        <v>652</v>
+      </c>
+      <c r="D493" s="46" t="inlineStr">
+        <is>
+          <t>35737</t>
+        </is>
+      </c>
+      <c r="E493" s="45" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F493" s="45" t="n">
+        <v>37</v>
+      </c>
+      <c r="G493" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H493" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="494" ht="20" customHeight="1">
+      <c r="A494" s="45" t="n">
+        <v>490</v>
+      </c>
+      <c r="B494" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C494" s="45" t="n">
+        <v>653</v>
+      </c>
+      <c r="D494" s="46" t="inlineStr">
+        <is>
+          <t>35741</t>
+        </is>
+      </c>
+      <c r="E494" s="45" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F494" s="45" t="n">
+        <v>32</v>
+      </c>
+      <c r="G494" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H494" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="495" ht="20" customHeight="1">
+      <c r="A495" s="45" t="n">
+        <v>491</v>
+      </c>
+      <c r="B495" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C495" s="45" t="n">
+        <v>641</v>
+      </c>
+      <c r="D495" s="46" t="inlineStr">
+        <is>
+          <t>35734</t>
+        </is>
+      </c>
+      <c r="E495" s="45" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F495" s="45" t="n">
+        <v>37</v>
+      </c>
+      <c r="G495" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H495" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="496" ht="20" customHeight="1">
+      <c r="A496" s="45" t="n">
+        <v>492</v>
+      </c>
+      <c r="B496" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C496" s="45" t="n">
+        <v>642</v>
+      </c>
+      <c r="D496" s="46" t="inlineStr">
+        <is>
+          <t>35662</t>
+        </is>
+      </c>
+      <c r="E496" s="45" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F496" s="45" t="n">
+        <v>34</v>
+      </c>
+      <c r="G496" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H496" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="497" ht="20" customHeight="1">
+      <c r="A497" s="45" t="n">
+        <v>493</v>
+      </c>
+      <c r="B497" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C497" s="45" t="n">
+        <v>638</v>
+      </c>
+      <c r="D497" s="46" t="inlineStr">
+        <is>
+          <t>35732</t>
+        </is>
+      </c>
+      <c r="E497" s="45" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F497" s="45" t="n">
+        <v>39</v>
+      </c>
+      <c r="G497" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H497" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="498" ht="20" customHeight="1">
+      <c r="A498" s="45" t="n">
+        <v>494</v>
+      </c>
+      <c r="B498" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C498" s="45" t="n">
+        <v>657</v>
+      </c>
+      <c r="D498" s="46" t="inlineStr">
+        <is>
+          <t>35740</t>
+        </is>
+      </c>
+      <c r="E498" s="45" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F498" s="45" t="n">
+        <v>39</v>
+      </c>
+      <c r="G498" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H498" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="499" ht="20" customHeight="1">
+      <c r="A499" s="45" t="n">
+        <v>495</v>
+      </c>
+      <c r="B499" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C499" s="45" t="n">
+        <v>640</v>
+      </c>
+      <c r="D499" s="46" t="inlineStr">
+        <is>
+          <t>35730</t>
+        </is>
+      </c>
+      <c r="E499" s="45" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F499" s="45" t="n">
+        <v>42</v>
+      </c>
+      <c r="G499" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H499" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="500" ht="20" customHeight="1">
+      <c r="A500" s="45" t="n">
+        <v>496</v>
+      </c>
+      <c r="B500" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C500" s="45" t="n">
+        <v>635</v>
+      </c>
+      <c r="D500" s="46" t="inlineStr">
+        <is>
+          <t>35663</t>
+        </is>
+      </c>
+      <c r="E500" s="45" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F500" s="45" t="n">
+        <v>44</v>
+      </c>
+      <c r="G500" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H500" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="501" ht="20" customHeight="1">
+      <c r="A501" s="45" t="n">
+        <v>497</v>
+      </c>
+      <c r="B501" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C501" s="45" t="n">
+        <v>636</v>
+      </c>
+      <c r="D501" s="46" t="inlineStr">
+        <is>
+          <t>35661</t>
+        </is>
+      </c>
+      <c r="E501" s="45" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="F501" s="45" t="n">
+        <v>42</v>
+      </c>
+      <c r="G501" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H501" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="502" ht="20" customHeight="1">
+      <c r="A502" s="45" t="n">
+        <v>498</v>
+      </c>
+      <c r="B502" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C502" s="45" t="n">
+        <v>634</v>
+      </c>
+      <c r="D502" s="46" t="inlineStr">
+        <is>
+          <t>35080</t>
+        </is>
+      </c>
+      <c r="E502" s="45" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F502" s="45" t="n">
+        <v>45</v>
+      </c>
+      <c r="G502" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H502" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="503" ht="20" customHeight="1">
+      <c r="A503" s="45" t="n">
+        <v>499</v>
+      </c>
+      <c r="B503" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C503" s="45" t="n">
+        <v>655</v>
+      </c>
+      <c r="D503" s="46" t="inlineStr">
+        <is>
+          <t>31991</t>
+        </is>
+      </c>
+      <c r="E503" s="45" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F503" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="G503" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H503" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="504" ht="20" customHeight="1">
+      <c r="A504" s="45" t="n">
+        <v>500</v>
+      </c>
+      <c r="B504" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C504" s="45" t="n">
+        <v>659</v>
+      </c>
+      <c r="D504" s="46" t="inlineStr">
+        <is>
+          <t>35084</t>
+        </is>
+      </c>
+      <c r="E504" s="45" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F504" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="G504" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H504" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="505" ht="20" customHeight="1">
+      <c r="A505" s="45" t="n">
+        <v>501</v>
+      </c>
+      <c r="B505" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C505" s="45" t="n">
+        <v>661</v>
+      </c>
+      <c r="D505" s="46" t="inlineStr">
+        <is>
+          <t>35085</t>
+        </is>
+      </c>
+      <c r="E505" s="45" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F505" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="G505" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H505" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="506" ht="20" customHeight="1">
+      <c r="A506" s="45" t="n">
+        <v>502</v>
+      </c>
+      <c r="B506" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C506" s="45" t="n">
+        <v>608</v>
+      </c>
+      <c r="D506" s="46" t="inlineStr">
+        <is>
+          <t>35340</t>
+        </is>
+      </c>
+      <c r="E506" s="45" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F506" s="45" t="n">
+        <v>42</v>
+      </c>
+      <c r="G506" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H506" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="507" ht="20" customHeight="1">
+      <c r="A507" s="45" t="n">
+        <v>503</v>
+      </c>
+      <c r="B507" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C507" s="45" t="n">
+        <v>633</v>
+      </c>
+      <c r="D507" s="46" t="inlineStr">
+        <is>
+          <t>35078</t>
+        </is>
+      </c>
+      <c r="E507" s="45" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F507" s="45" t="n">
+        <v>36</v>
+      </c>
+      <c r="G507" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H507" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="508" ht="20" customHeight="1">
+      <c r="A508" s="45" t="n">
+        <v>504</v>
+      </c>
+      <c r="B508" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C508" s="45" t="n">
+        <v>632</v>
+      </c>
+      <c r="D508" s="46" t="inlineStr">
+        <is>
+          <t>35079</t>
+        </is>
+      </c>
+      <c r="E508" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F508" s="45" t="n">
+        <v>37</v>
+      </c>
+      <c r="G508" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H508" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="509" ht="20" customHeight="1">
+      <c r="A509" s="45" t="n">
+        <v>505</v>
+      </c>
+      <c r="B509" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C509" s="45" t="n">
+        <v>654</v>
+      </c>
+      <c r="D509" s="46" t="inlineStr">
+        <is>
+          <t>35081</t>
+        </is>
+      </c>
+      <c r="E509" s="45" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F509" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="G509" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H509" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="510" ht="20" customHeight="1">
+      <c r="A510" s="45" t="n">
+        <v>506</v>
+      </c>
+      <c r="B510" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C510" s="45" t="n">
+        <v>631</v>
+      </c>
+      <c r="D510" s="46" t="inlineStr">
+        <is>
+          <t>35087</t>
+        </is>
+      </c>
+      <c r="E510" s="45" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F510" s="45" t="n">
+        <v>34</v>
+      </c>
+      <c r="G510" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H510" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="511" ht="20" customHeight="1">
+      <c r="A511" s="45" t="n">
+        <v>507</v>
+      </c>
+      <c r="B511" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C511" s="45" t="n">
+        <v>601</v>
+      </c>
+      <c r="D511" s="46" t="inlineStr">
+        <is>
+          <t>31993</t>
+        </is>
+      </c>
+      <c r="E511" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F511" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="G511" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H511" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="512" ht="20" customHeight="1">
+      <c r="A512" s="45" t="n">
+        <v>508</v>
+      </c>
+      <c r="B512" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C512" s="45" t="n">
+        <v>602</v>
+      </c>
+      <c r="D512" s="46" t="inlineStr">
+        <is>
+          <t>35339</t>
+        </is>
+      </c>
+      <c r="E512" s="45" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F512" s="45" t="n">
+        <v>48</v>
+      </c>
+      <c r="G512" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H512" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="513" ht="20" customHeight="1">
+      <c r="A513" s="45" t="n">
+        <v>509</v>
+      </c>
+      <c r="B513" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C513" s="45" t="n">
+        <v>658</v>
+      </c>
+      <c r="D513" s="46" t="inlineStr">
+        <is>
+          <t>35083</t>
+        </is>
+      </c>
+      <c r="E513" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F513" s="45" t="n">
+        <v>33</v>
+      </c>
+      <c r="G513" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H513" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="514" ht="20" customHeight="1">
+      <c r="A514" s="45" t="n">
+        <v>510</v>
+      </c>
+      <c r="B514" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C514" s="45" t="n">
+        <v>660</v>
+      </c>
+      <c r="D514" s="46" t="inlineStr">
+        <is>
+          <t>35086</t>
+        </is>
+      </c>
+      <c r="E514" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F514" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="G514" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H514" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="515" ht="20" customHeight="1">
+      <c r="A515" s="45" t="n">
+        <v>511</v>
+      </c>
+      <c r="B515" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C515" s="45" t="n">
+        <v>630</v>
+      </c>
+      <c r="D515" s="46" t="inlineStr">
+        <is>
+          <t>35082</t>
+        </is>
+      </c>
+      <c r="E515" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F515" s="45" t="n">
+        <v>30</v>
+      </c>
+      <c r="G515" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H515" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="516" ht="20" customHeight="1">
+      <c r="A516" s="45" t="n">
+        <v>512</v>
+      </c>
+      <c r="B516" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C516" s="45" t="n">
+        <v>625</v>
+      </c>
+      <c r="D516" s="46" t="inlineStr">
+        <is>
+          <t>35088</t>
+        </is>
+      </c>
+      <c r="E516" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F516" s="45" t="n">
+        <v>44</v>
+      </c>
+      <c r="G516" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H516" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="517" ht="20" customHeight="1">
+      <c r="A517" s="45" t="n">
+        <v>513</v>
+      </c>
+      <c r="B517" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C517" s="45" t="n">
+        <v>626</v>
+      </c>
+      <c r="D517" s="46" t="inlineStr">
+        <is>
+          <t>31989</t>
+        </is>
+      </c>
+      <c r="E517" s="45" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F517" s="45" t="n">
+        <v>43</v>
+      </c>
+      <c r="G517" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H517" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="518" ht="20" customHeight="1">
+      <c r="A518" s="45" t="n">
+        <v>514</v>
+      </c>
+      <c r="B518" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C518" s="45" t="n">
+        <v>627</v>
+      </c>
+      <c r="D518" s="46" t="inlineStr">
+        <is>
+          <t>31990</t>
+        </is>
+      </c>
+      <c r="E518" s="45" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F518" s="45" t="n">
+        <v>41</v>
+      </c>
+      <c r="G518" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H518" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="519" ht="20" customHeight="1">
+      <c r="A519" s="45" t="n">
+        <v>515</v>
+      </c>
+      <c r="B519" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C519" s="45" t="n">
+        <v>628</v>
+      </c>
+      <c r="D519" s="46" t="inlineStr">
+        <is>
+          <t>31995</t>
+        </is>
+      </c>
+      <c r="E519" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F519" s="45" t="n">
+        <v>40</v>
+      </c>
+      <c r="G519" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H519" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="520" ht="20" customHeight="1">
+      <c r="A520" s="45" t="n">
+        <v>516</v>
+      </c>
+      <c r="B520" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C520" s="45" t="n">
+        <v>656</v>
+      </c>
+      <c r="D520" s="46" t="inlineStr">
+        <is>
+          <t>31992</t>
+        </is>
+      </c>
+      <c r="E520" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F520" s="45" t="n">
+        <v>31</v>
+      </c>
+      <c r="G520" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H520" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="521" ht="20" customHeight="1">
+      <c r="A521" s="45" t="n">
+        <v>517</v>
+      </c>
+      <c r="B521" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C521" s="45" t="n">
+        <v>629</v>
+      </c>
+      <c r="D521" s="46" t="inlineStr">
+        <is>
+          <t>31994</t>
+        </is>
+      </c>
+      <c r="E521" s="45" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F521" s="45" t="n">
+        <v>39</v>
+      </c>
+      <c r="G521" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H521" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="522" ht="20" customHeight="1">
+      <c r="A522" s="45" t="n">
+        <v>518</v>
+      </c>
+      <c r="B522" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C522" s="45" t="n">
+        <v>662</v>
+      </c>
+      <c r="D522" s="46" t="inlineStr">
+        <is>
+          <t>35341</t>
+        </is>
+      </c>
+      <c r="E522" s="45" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F522" s="45" t="n">
+        <v>45</v>
+      </c>
+      <c r="G522" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H522" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="523" ht="22" customHeight="1">
+      <c r="A523" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL KESELURUHAN (518 BAL)</t>
+        </is>
+      </c>
+      <c r="B523" s="35" t="n"/>
+      <c r="C523" s="35" t="n"/>
+      <c r="D523" s="35" t="n"/>
+      <c r="E523" s="35" t="n"/>
+      <c r="F523" s="35">
+        <f>SUM(F5:F522)</f>
         <v/>
       </c>
-      <c r="G482" s="35">
-        <f>COUNTA(A5:A481) &amp; " Bal"</f>
-        <v/>
-      </c>
-      <c r="H482" s="37" t="n"/>
+      <c r="G523" s="35" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="H523" s="35" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A482:E482"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A463:E463"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A523:E523"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21070,9 +22612,9 @@
           <t>TOTAL (19 BAL)</t>
         </is>
       </c>
-      <c r="B24" s="36" t="n"/>
-      <c r="C24" s="36" t="n"/>
-      <c r="D24" s="36" t="n"/>
+      <c r="B24" s="42" t="n"/>
+      <c r="C24" s="42" t="n"/>
+      <c r="D24" s="43" t="n"/>
       <c r="E24" s="35">
         <f>SUM(E5:E23)</f>
         <v/>
@@ -21085,6 +22627,1376 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A24:D24"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="47" t="inlineStr">
+        <is>
+          <t>T.B.K JH • REKAPITULASI HARIAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="48" t="inlineStr">
+        <is>
+          <t>Data Bal Gudang Induk Tanggal: 1 September 2026 (Selasa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>No Gud</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>Nomor Barkot</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="35" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="45" t="n">
+        <v>649</v>
+      </c>
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>33863</t>
+        </is>
+      </c>
+      <c r="D5" s="45" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E5" s="45" t="n">
+        <v>38</v>
+      </c>
+      <c r="F5" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="45" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="45" t="n">
+        <v>647</v>
+      </c>
+      <c r="C6" s="46" t="inlineStr">
+        <is>
+          <t>33862</t>
+        </is>
+      </c>
+      <c r="D6" s="45" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E6" s="45" t="n">
+        <v>39</v>
+      </c>
+      <c r="F6" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="45" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="45" t="n">
+        <v>648</v>
+      </c>
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>33861</t>
+        </is>
+      </c>
+      <c r="D7" s="45" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E7" s="45" t="n">
+        <v>40</v>
+      </c>
+      <c r="F7" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G7" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="45" t="n">
+        <v>644</v>
+      </c>
+      <c r="C8" s="46" t="inlineStr">
+        <is>
+          <t>35733</t>
+        </is>
+      </c>
+      <c r="D8" s="45" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E8" s="45" t="n">
+        <v>47</v>
+      </c>
+      <c r="F8" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="45" t="n">
+        <v>646</v>
+      </c>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>33860</t>
+        </is>
+      </c>
+      <c r="D9" s="45" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E9" s="45" t="n">
+        <v>42</v>
+      </c>
+      <c r="F9" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="45" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="45" t="n">
+        <v>645</v>
+      </c>
+      <c r="C10" s="46" t="inlineStr">
+        <is>
+          <t>35735</t>
+        </is>
+      </c>
+      <c r="D10" s="45" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E10" s="45" t="n">
+        <v>43</v>
+      </c>
+      <c r="F10" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="45" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="45" t="n">
+        <v>643</v>
+      </c>
+      <c r="C11" s="46" t="inlineStr">
+        <is>
+          <t>35736</t>
+        </is>
+      </c>
+      <c r="D11" s="45" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E11" s="45" t="n">
+        <v>46</v>
+      </c>
+      <c r="F11" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="45" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="45" t="n">
+        <v>637</v>
+      </c>
+      <c r="C12" s="46" t="inlineStr">
+        <is>
+          <t>35729</t>
+        </is>
+      </c>
+      <c r="D12" s="45" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E12" s="45" t="n">
+        <v>49</v>
+      </c>
+      <c r="F12" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="45" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="45" t="n">
+        <v>639</v>
+      </c>
+      <c r="C13" s="46" t="inlineStr">
+        <is>
+          <t>35731</t>
+        </is>
+      </c>
+      <c r="D13" s="45" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E13" s="45" t="n">
+        <v>41</v>
+      </c>
+      <c r="F13" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="45" t="n">
+        <v>650</v>
+      </c>
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>35739</t>
+        </is>
+      </c>
+      <c r="D14" s="45" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E14" s="45" t="n">
+        <v>30</v>
+      </c>
+      <c r="F14" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="45" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="45" t="n">
+        <v>651</v>
+      </c>
+      <c r="C15" s="46" t="inlineStr">
+        <is>
+          <t>35738</t>
+        </is>
+      </c>
+      <c r="D15" s="45" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E15" s="45" t="n">
+        <v>41</v>
+      </c>
+      <c r="F15" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="45" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="45" t="n">
+        <v>652</v>
+      </c>
+      <c r="C16" s="46" t="inlineStr">
+        <is>
+          <t>35737</t>
+        </is>
+      </c>
+      <c r="D16" s="45" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E16" s="45" t="n">
+        <v>37</v>
+      </c>
+      <c r="F16" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="45" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="45" t="n">
+        <v>653</v>
+      </c>
+      <c r="C17" s="46" t="inlineStr">
+        <is>
+          <t>35741</t>
+        </is>
+      </c>
+      <c r="D17" s="45" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E17" s="45" t="n">
+        <v>32</v>
+      </c>
+      <c r="F17" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="45" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="45" t="n">
+        <v>641</v>
+      </c>
+      <c r="C18" s="46" t="inlineStr">
+        <is>
+          <t>35734</t>
+        </is>
+      </c>
+      <c r="D18" s="45" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E18" s="45" t="n">
+        <v>37</v>
+      </c>
+      <c r="F18" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="45" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="45" t="n">
+        <v>642</v>
+      </c>
+      <c r="C19" s="46" t="inlineStr">
+        <is>
+          <t>35662</t>
+        </is>
+      </c>
+      <c r="D19" s="45" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E19" s="45" t="n">
+        <v>34</v>
+      </c>
+      <c r="F19" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="45" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="45" t="n">
+        <v>638</v>
+      </c>
+      <c r="C20" s="46" t="inlineStr">
+        <is>
+          <t>35732</t>
+        </is>
+      </c>
+      <c r="D20" s="45" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E20" s="45" t="n">
+        <v>39</v>
+      </c>
+      <c r="F20" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="45" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="45" t="n">
+        <v>657</v>
+      </c>
+      <c r="C21" s="46" t="inlineStr">
+        <is>
+          <t>35740</t>
+        </is>
+      </c>
+      <c r="D21" s="45" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E21" s="45" t="n">
+        <v>39</v>
+      </c>
+      <c r="F21" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="45" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="45" t="n">
+        <v>640</v>
+      </c>
+      <c r="C22" s="46" t="inlineStr">
+        <is>
+          <t>35730</t>
+        </is>
+      </c>
+      <c r="D22" s="45" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E22" s="45" t="n">
+        <v>42</v>
+      </c>
+      <c r="F22" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="45" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="45" t="n">
+        <v>635</v>
+      </c>
+      <c r="C23" s="46" t="inlineStr">
+        <is>
+          <t>35663</t>
+        </is>
+      </c>
+      <c r="D23" s="45" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E23" s="45" t="n">
+        <v>44</v>
+      </c>
+      <c r="F23" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="45" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="45" t="n">
+        <v>636</v>
+      </c>
+      <c r="C24" s="46" t="inlineStr">
+        <is>
+          <t>35661</t>
+        </is>
+      </c>
+      <c r="D24" s="45" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="E24" s="45" t="n">
+        <v>42</v>
+      </c>
+      <c r="F24" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="45" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="45" t="n">
+        <v>634</v>
+      </c>
+      <c r="C25" s="46" t="inlineStr">
+        <is>
+          <t>35080</t>
+        </is>
+      </c>
+      <c r="D25" s="45" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E25" s="45" t="n">
+        <v>45</v>
+      </c>
+      <c r="F25" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G25" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="45" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="45" t="n">
+        <v>655</v>
+      </c>
+      <c r="C26" s="46" t="inlineStr">
+        <is>
+          <t>31991</t>
+        </is>
+      </c>
+      <c r="D26" s="45" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E26" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="F26" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G26" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="45" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="45" t="n">
+        <v>659</v>
+      </c>
+      <c r="C27" s="46" t="inlineStr">
+        <is>
+          <t>35084</t>
+        </is>
+      </c>
+      <c r="D27" s="45" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E27" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="F27" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G27" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="45" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="45" t="n">
+        <v>661</v>
+      </c>
+      <c r="C28" s="46" t="inlineStr">
+        <is>
+          <t>35085</t>
+        </is>
+      </c>
+      <c r="D28" s="45" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E28" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="F28" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G28" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="45" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="45" t="n">
+        <v>608</v>
+      </c>
+      <c r="C29" s="46" t="inlineStr">
+        <is>
+          <t>35340</t>
+        </is>
+      </c>
+      <c r="D29" s="45" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>42</v>
+      </c>
+      <c r="F29" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G29" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="45" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="45" t="n">
+        <v>633</v>
+      </c>
+      <c r="C30" s="46" t="inlineStr">
+        <is>
+          <t>35078</t>
+        </is>
+      </c>
+      <c r="D30" s="45" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E30" s="45" t="n">
+        <v>36</v>
+      </c>
+      <c r="F30" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G30" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="45" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="45" t="n">
+        <v>632</v>
+      </c>
+      <c r="C31" s="46" t="inlineStr">
+        <is>
+          <t>35079</t>
+        </is>
+      </c>
+      <c r="D31" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E31" s="45" t="n">
+        <v>37</v>
+      </c>
+      <c r="F31" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G31" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="45" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="45" t="n">
+        <v>654</v>
+      </c>
+      <c r="C32" s="46" t="inlineStr">
+        <is>
+          <t>35081</t>
+        </is>
+      </c>
+      <c r="D32" s="45" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E32" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="F32" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G32" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="45" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="45" t="n">
+        <v>631</v>
+      </c>
+      <c r="C33" s="46" t="inlineStr">
+        <is>
+          <t>35087</t>
+        </is>
+      </c>
+      <c r="D33" s="45" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E33" s="45" t="n">
+        <v>34</v>
+      </c>
+      <c r="F33" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G33" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="45" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="45" t="n">
+        <v>601</v>
+      </c>
+      <c r="C34" s="46" t="inlineStr">
+        <is>
+          <t>31993</t>
+        </is>
+      </c>
+      <c r="D34" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E34" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="F34" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G34" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="45" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="45" t="n">
+        <v>602</v>
+      </c>
+      <c r="C35" s="46" t="inlineStr">
+        <is>
+          <t>35339</t>
+        </is>
+      </c>
+      <c r="D35" s="45" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E35" s="45" t="n">
+        <v>48</v>
+      </c>
+      <c r="F35" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G35" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="45" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="45" t="n">
+        <v>658</v>
+      </c>
+      <c r="C36" s="46" t="inlineStr">
+        <is>
+          <t>35083</t>
+        </is>
+      </c>
+      <c r="D36" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E36" s="45" t="n">
+        <v>33</v>
+      </c>
+      <c r="F36" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G36" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="45" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="45" t="n">
+        <v>660</v>
+      </c>
+      <c r="C37" s="46" t="inlineStr">
+        <is>
+          <t>35086</t>
+        </is>
+      </c>
+      <c r="D37" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E37" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="F37" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G37" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="45" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="45" t="n">
+        <v>630</v>
+      </c>
+      <c r="C38" s="46" t="inlineStr">
+        <is>
+          <t>35082</t>
+        </is>
+      </c>
+      <c r="D38" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E38" s="45" t="n">
+        <v>30</v>
+      </c>
+      <c r="F38" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G38" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="45" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="45" t="n">
+        <v>625</v>
+      </c>
+      <c r="C39" s="46" t="inlineStr">
+        <is>
+          <t>35088</t>
+        </is>
+      </c>
+      <c r="D39" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E39" s="45" t="n">
+        <v>44</v>
+      </c>
+      <c r="F39" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G39" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="45" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="45" t="n">
+        <v>626</v>
+      </c>
+      <c r="C40" s="46" t="inlineStr">
+        <is>
+          <t>31989</t>
+        </is>
+      </c>
+      <c r="D40" s="45" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E40" s="45" t="n">
+        <v>43</v>
+      </c>
+      <c r="F40" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G40" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="45" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="45" t="n">
+        <v>627</v>
+      </c>
+      <c r="C41" s="46" t="inlineStr">
+        <is>
+          <t>31990</t>
+        </is>
+      </c>
+      <c r="D41" s="45" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E41" s="45" t="n">
+        <v>41</v>
+      </c>
+      <c r="F41" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G41" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="45" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="45" t="n">
+        <v>628</v>
+      </c>
+      <c r="C42" s="46" t="inlineStr">
+        <is>
+          <t>31995</t>
+        </is>
+      </c>
+      <c r="D42" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E42" s="45" t="n">
+        <v>40</v>
+      </c>
+      <c r="F42" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G42" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="45" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="45" t="n">
+        <v>656</v>
+      </c>
+      <c r="C43" s="46" t="inlineStr">
+        <is>
+          <t>31992</t>
+        </is>
+      </c>
+      <c r="D43" s="45" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E43" s="45" t="n">
+        <v>31</v>
+      </c>
+      <c r="F43" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G43" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="45" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="45" t="n">
+        <v>629</v>
+      </c>
+      <c r="C44" s="46" t="inlineStr">
+        <is>
+          <t>31994</t>
+        </is>
+      </c>
+      <c r="D44" s="45" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E44" s="45" t="n">
+        <v>39</v>
+      </c>
+      <c r="F44" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G44" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="45" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="45" t="n">
+        <v>662</v>
+      </c>
+      <c r="C45" s="46" t="inlineStr">
+        <is>
+          <t>35341</t>
+        </is>
+      </c>
+      <c r="D45" s="45" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E45" s="45" t="n">
+        <v>45</v>
+      </c>
+      <c r="F45" s="45" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G45" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL (41 BAL)</t>
+        </is>
+      </c>
+      <c r="B46" s="35" t="n"/>
+      <c r="C46" s="35" t="n"/>
+      <c r="D46" s="35" t="n"/>
+      <c r="E46" s="35">
+        <f>SUM(E5:E45)</f>
+        <v/>
+      </c>
+      <c r="F46" s="35" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G46" s="35" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A46:D46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21096,7 +24008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21388,11 +24300,7 @@
       <c r="A14" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="32" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
+      <c r="B14" s="43" t="n"/>
       <c r="C14" s="32" t="inlineStr">
         <is>
           <t>Senin</t>
@@ -21412,37 +24320,67 @@
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="35" t="inlineStr">
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="44" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C15" s="45" t="inlineStr">
+        <is>
+          <t>Selasa</t>
+        </is>
+      </c>
+      <c r="D15" s="44" t="n">
+        <v>41</v>
+      </c>
+      <c r="E15" s="44" t="n">
+        <v>1690</v>
+      </c>
+      <c r="F15" s="44" t="n">
+        <v>41.22</v>
+      </c>
+      <c r="G15" s="44" t="inlineStr">
+        <is>
+          <t>601 - 662</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="35" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B15" s="36" t="n"/>
-      <c r="C15" s="36" t="n"/>
-      <c r="D15" s="35">
-        <f>SUM(D5:D14)</f>
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="35" t="n"/>
+      <c r="D16" s="35">
+        <f>SUM(D5:D15)</f>
         <v/>
       </c>
-      <c r="E15" s="35">
-        <f>SUM(E5:E14)</f>
+      <c r="E16" s="35">
+        <f>SUM(E5:E15)</f>
         <v/>
       </c>
-      <c r="F15" s="35">
-        <f>SUM(F5:F14)</f>
+      <c r="F16" s="35">
+        <f>AVERAGE(F5:F15)</f>
         <v/>
       </c>
-      <c r="G15" s="35">
-        <f>SUM(G5:G14)</f>
-        <v/>
+      <c r="G16" s="35" t="inlineStr">
+        <is>
+          <t>64 - 662</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data 3 September 2026 (25 bal), rekap buku grade induk, dan sinkronisasi Supabase
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -21,6 +21,7 @@
     <sheet name="31 Agustus" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="1 September" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="2 September" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="3 September" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +33,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;kg&quot;"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -158,6 +159,20 @@
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -221,7 +236,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -379,11 +394,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -534,6 +563,24 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -901,7 +948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H551"/>
+  <dimension ref="A1:H576"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -924,7 +971,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Laporan Lengkap No Gudang, Nomor Barcode, Grade, dan Berat (Kg) Semua Tanggal (21 Agustus - 2 September 2026)</t>
+          <t>Laporan Lengkap No Gudang, Nomor Barcode, Grade, dan Berat (Kg) Semua Tanggal (21 Agustus - 3 September 2026)</t>
         </is>
       </c>
     </row>
@@ -17364,24 +17411,10 @@
       <c r="A463" s="49" t="n">
         <v>459</v>
       </c>
-      <c r="B463" s="49" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C463" s="49" t="n">
-        <v>605</v>
-      </c>
-      <c r="D463" s="50" t="inlineStr">
-        <is>
-          <t>34953</t>
-        </is>
-      </c>
-      <c r="E463" s="49" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
+      <c r="B463" s="42" t="n"/>
+      <c r="C463" s="42" t="n"/>
+      <c r="D463" s="42" t="n"/>
+      <c r="E463" s="43" t="n"/>
       <c r="F463" s="51" t="n">
         <v>38</v>
       </c>
@@ -19524,24 +19557,10 @@
       <c r="A523" s="49" t="n">
         <v>519</v>
       </c>
-      <c r="B523" s="49" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="C523" s="49" t="n">
-        <v>663</v>
-      </c>
-      <c r="D523" s="50" t="inlineStr">
-        <is>
-          <t>35999</t>
-        </is>
-      </c>
-      <c r="E523" s="49" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
-      </c>
+      <c r="B523" s="42" t="n"/>
+      <c r="C523" s="42" t="n"/>
+      <c r="D523" s="42" t="n"/>
+      <c r="E523" s="43" t="n"/>
       <c r="F523" s="51" t="n">
         <v>42</v>
       </c>
@@ -20528,34 +20547,809 @@
         </is>
       </c>
     </row>
-    <row r="551">
-      <c r="A551" s="53" t="inlineStr">
-        <is>
-          <t>TOTAL KESELURUHAN (546 BAL)</t>
-        </is>
-      </c>
-      <c r="B551" s="53" t="n"/>
-      <c r="C551" s="53" t="n"/>
-      <c r="D551" s="53" t="n"/>
-      <c r="E551" s="53" t="n"/>
-      <c r="F551" s="53">
-        <f>SUM(F5:F550)</f>
+    <row r="551" ht="20" customHeight="1">
+      <c r="A551" s="49" t="n">
+        <v>547</v>
+      </c>
+      <c r="B551" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C551" s="49" t="n">
+        <v>698</v>
+      </c>
+      <c r="D551" s="50" t="inlineStr">
+        <is>
+          <t>35489</t>
+        </is>
+      </c>
+      <c r="E551" s="49" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F551" s="51" t="n">
+        <v>33</v>
+      </c>
+      <c r="G551" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H551" s="53" t="inlineStr"/>
+    </row>
+    <row r="552" ht="20" customHeight="1">
+      <c r="A552" s="49" t="n">
+        <v>548</v>
+      </c>
+      <c r="B552" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C552" s="49" t="n">
+        <v>699</v>
+      </c>
+      <c r="D552" s="50" t="inlineStr">
+        <is>
+          <t>35490</t>
+        </is>
+      </c>
+      <c r="E552" s="49" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F552" s="51" t="n">
+        <v>50</v>
+      </c>
+      <c r="G552" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="553" ht="20" customHeight="1">
+      <c r="A553" s="49" t="n">
+        <v>549</v>
+      </c>
+      <c r="B553" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C553" s="49" t="n">
+        <v>697</v>
+      </c>
+      <c r="D553" s="50" t="inlineStr">
+        <is>
+          <t>39096</t>
+        </is>
+      </c>
+      <c r="E553" s="49" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F553" s="51" t="n">
+        <v>44</v>
+      </c>
+      <c r="G553" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="554" ht="20" customHeight="1">
+      <c r="A554" s="49" t="n">
+        <v>550</v>
+      </c>
+      <c r="B554" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C554" s="49" t="n">
+        <v>696</v>
+      </c>
+      <c r="D554" s="50" t="inlineStr">
+        <is>
+          <t>39097</t>
+        </is>
+      </c>
+      <c r="E554" s="49" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F554" s="51" t="n">
+        <v>39</v>
+      </c>
+      <c r="G554" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="555" ht="20" customHeight="1">
+      <c r="A555" s="49" t="n">
+        <v>551</v>
+      </c>
+      <c r="B555" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C555" s="49" t="n">
+        <v>692</v>
+      </c>
+      <c r="D555" s="50" t="inlineStr">
+        <is>
+          <t>39780</t>
+        </is>
+      </c>
+      <c r="E555" s="49" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F555" s="51" t="n">
+        <v>35</v>
+      </c>
+      <c r="G555" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="556" ht="20" customHeight="1">
+      <c r="A556" s="49" t="n">
+        <v>552</v>
+      </c>
+      <c r="B556" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C556" s="49" t="n">
+        <v>693</v>
+      </c>
+      <c r="D556" s="50" t="inlineStr">
+        <is>
+          <t>39098</t>
+        </is>
+      </c>
+      <c r="E556" s="49" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F556" s="51" t="n">
+        <v>37</v>
+      </c>
+      <c r="G556" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="557" ht="20" customHeight="1">
+      <c r="A557" s="49" t="n">
+        <v>553</v>
+      </c>
+      <c r="B557" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C557" s="49" t="n">
+        <v>694</v>
+      </c>
+      <c r="D557" s="50" t="inlineStr">
+        <is>
+          <t>39092</t>
+        </is>
+      </c>
+      <c r="E557" s="49" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F557" s="51" t="n">
+        <v>38</v>
+      </c>
+      <c r="G557" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="558" ht="20" customHeight="1">
+      <c r="A558" s="49" t="n">
+        <v>554</v>
+      </c>
+      <c r="B558" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C558" s="49" t="n">
+        <v>695</v>
+      </c>
+      <c r="D558" s="50" t="inlineStr">
+        <is>
+          <t>39091</t>
+        </is>
+      </c>
+      <c r="E558" s="49" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F558" s="51" t="n">
+        <v>43</v>
+      </c>
+      <c r="G558" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="559" ht="20" customHeight="1">
+      <c r="A559" s="49" t="n">
+        <v>555</v>
+      </c>
+      <c r="B559" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C559" s="49" t="n">
+        <v>688</v>
+      </c>
+      <c r="D559" s="50" t="inlineStr">
+        <is>
+          <t>39095</t>
+        </is>
+      </c>
+      <c r="E559" s="49" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F559" s="51" t="n">
+        <v>41</v>
+      </c>
+      <c r="G559" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="560" ht="20" customHeight="1">
+      <c r="A560" s="49" t="n">
+        <v>556</v>
+      </c>
+      <c r="B560" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C560" s="49" t="n">
+        <v>700</v>
+      </c>
+      <c r="D560" s="50" t="inlineStr">
+        <is>
+          <t>39779</t>
+        </is>
+      </c>
+      <c r="E560" s="49" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F560" s="51" t="n">
+        <v>37</v>
+      </c>
+      <c r="G560" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="561" ht="20" customHeight="1">
+      <c r="A561" s="49" t="n">
+        <v>557</v>
+      </c>
+      <c r="B561" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C561" s="49" t="n">
+        <v>691</v>
+      </c>
+      <c r="D561" s="50" t="inlineStr">
+        <is>
+          <t>39778</t>
+        </is>
+      </c>
+      <c r="E561" s="49" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F561" s="51" t="n">
+        <v>35</v>
+      </c>
+      <c r="G561" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="562" ht="20" customHeight="1">
+      <c r="A562" s="49" t="n">
+        <v>558</v>
+      </c>
+      <c r="B562" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C562" s="49" t="n">
+        <v>701</v>
+      </c>
+      <c r="D562" s="50" t="inlineStr">
+        <is>
+          <t>39776</t>
+        </is>
+      </c>
+      <c r="E562" s="49" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F562" s="51" t="n">
+        <v>35</v>
+      </c>
+      <c r="G562" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="563" ht="20" customHeight="1">
+      <c r="A563" s="49" t="n">
+        <v>559</v>
+      </c>
+      <c r="B563" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C563" s="49" t="n">
+        <v>689</v>
+      </c>
+      <c r="D563" s="50" t="inlineStr">
+        <is>
+          <t>39094</t>
+        </is>
+      </c>
+      <c r="E563" s="49" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F563" s="51" t="n">
+        <v>38</v>
+      </c>
+      <c r="G563" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="564" ht="20" customHeight="1">
+      <c r="A564" s="49" t="n">
+        <v>560</v>
+      </c>
+      <c r="B564" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C564" s="49" t="n">
+        <v>702</v>
+      </c>
+      <c r="D564" s="50" t="inlineStr">
+        <is>
+          <t>39093</t>
+        </is>
+      </c>
+      <c r="E564" s="49" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F564" s="51" t="n">
+        <v>50</v>
+      </c>
+      <c r="G564" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="565" ht="20" customHeight="1">
+      <c r="A565" s="49" t="n">
+        <v>561</v>
+      </c>
+      <c r="B565" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C565" s="49" t="n">
+        <v>690</v>
+      </c>
+      <c r="D565" s="50" t="inlineStr">
+        <is>
+          <t>39777</t>
+        </is>
+      </c>
+      <c r="E565" s="49" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F565" s="51" t="n">
+        <v>35</v>
+      </c>
+      <c r="G565" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="566" ht="20" customHeight="1">
+      <c r="A566" s="49" t="n">
+        <v>562</v>
+      </c>
+      <c r="B566" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C566" s="49" t="n">
+        <v>703</v>
+      </c>
+      <c r="D566" s="50" t="inlineStr">
+        <is>
+          <t>39089</t>
+        </is>
+      </c>
+      <c r="E566" s="49" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F566" s="51" t="n">
+        <v>45</v>
+      </c>
+      <c r="G566" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="567" ht="20" customHeight="1">
+      <c r="A567" s="49" t="n">
+        <v>563</v>
+      </c>
+      <c r="B567" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C567" s="49" t="n">
+        <v>687</v>
+      </c>
+      <c r="D567" s="50" t="inlineStr">
+        <is>
+          <t>39090</t>
+        </is>
+      </c>
+      <c r="E567" s="49" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F567" s="51" t="n">
+        <v>41</v>
+      </c>
+      <c r="G567" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="568" ht="20" customHeight="1">
+      <c r="A568" s="49" t="n">
+        <v>564</v>
+      </c>
+      <c r="B568" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C568" s="49" t="n">
+        <v>704</v>
+      </c>
+      <c r="D568" s="50" t="inlineStr">
+        <is>
+          <t>39088</t>
+        </is>
+      </c>
+      <c r="E568" s="49" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F568" s="51" t="n">
+        <v>32</v>
+      </c>
+      <c r="G568" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="569" ht="20" customHeight="1">
+      <c r="A569" s="49" t="n">
+        <v>565</v>
+      </c>
+      <c r="B569" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C569" s="49" t="n">
+        <v>705</v>
+      </c>
+      <c r="D569" s="50" t="inlineStr">
+        <is>
+          <t>39775</t>
+        </is>
+      </c>
+      <c r="E569" s="49" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F569" s="51" t="n">
+        <v>34</v>
+      </c>
+      <c r="G569" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="570" ht="20" customHeight="1">
+      <c r="A570" s="49" t="n">
+        <v>566</v>
+      </c>
+      <c r="B570" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C570" s="49" t="n">
+        <v>706</v>
+      </c>
+      <c r="D570" s="50" t="inlineStr">
+        <is>
+          <t>39774</t>
+        </is>
+      </c>
+      <c r="E570" s="49" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F570" s="51" t="n">
+        <v>40</v>
+      </c>
+      <c r="G570" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="571" ht="20" customHeight="1">
+      <c r="A571" s="49" t="n">
+        <v>567</v>
+      </c>
+      <c r="B571" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C571" s="49" t="n">
+        <v>707</v>
+      </c>
+      <c r="D571" s="50" t="inlineStr">
+        <is>
+          <t>39086</t>
+        </is>
+      </c>
+      <c r="E571" s="49" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F571" s="51" t="n">
+        <v>48</v>
+      </c>
+      <c r="G571" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="572" ht="20" customHeight="1">
+      <c r="A572" s="49" t="n">
+        <v>568</v>
+      </c>
+      <c r="B572" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C572" s="49" t="n">
+        <v>708</v>
+      </c>
+      <c r="D572" s="50" t="inlineStr">
+        <is>
+          <t>39084</t>
+        </is>
+      </c>
+      <c r="E572" s="49" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F572" s="51" t="n">
+        <v>35</v>
+      </c>
+      <c r="G572" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="573" ht="20" customHeight="1">
+      <c r="A573" s="49" t="n">
+        <v>569</v>
+      </c>
+      <c r="B573" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C573" s="49" t="n">
+        <v>709</v>
+      </c>
+      <c r="D573" s="50" t="inlineStr">
+        <is>
+          <t>39085</t>
+        </is>
+      </c>
+      <c r="E573" s="49" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F573" s="51" t="n">
+        <v>39</v>
+      </c>
+      <c r="G573" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="574" ht="20" customHeight="1">
+      <c r="A574" s="49" t="n">
+        <v>570</v>
+      </c>
+      <c r="B574" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C574" s="49" t="n">
+        <v>710</v>
+      </c>
+      <c r="D574" s="50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E574" s="49" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F574" s="51" t="n">
+        <v>31</v>
+      </c>
+      <c r="G574" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="575" ht="20" customHeight="1">
+      <c r="A575" s="49" t="n">
+        <v>571</v>
+      </c>
+      <c r="B575" s="49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C575" s="49" t="n">
+        <v>711</v>
+      </c>
+      <c r="D575" s="50" t="inlineStr">
+        <is>
+          <t>39087</t>
+        </is>
+      </c>
+      <c r="E575" s="49" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F575" s="51" t="n">
+        <v>38</v>
+      </c>
+      <c r="G575" s="49" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="576" ht="22" customHeight="1">
+      <c r="A576" s="56" t="inlineStr">
+        <is>
+          <t>TOTAL KESELURUHAN (571 BAL)</t>
+        </is>
+      </c>
+      <c r="B576" s="56" t="n"/>
+      <c r="C576" s="56" t="n"/>
+      <c r="D576" s="56" t="n"/>
+      <c r="E576" s="56" t="n"/>
+      <c r="F576" s="56">
+        <f>SUM(F5:F575)</f>
         <v/>
       </c>
-      <c r="G551" s="53" t="inlineStr">
+      <c r="G576" s="56" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
       </c>
-      <c r="H551" s="53" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A551:E551"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A463:E463"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A523:E523"/>
+    <mergeCell ref="A576:E576"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26013,9 +26807,9 @@
           <t>TOTAL (28 BAL)</t>
         </is>
       </c>
-      <c r="B33" s="53" t="n"/>
-      <c r="C33" s="53" t="n"/>
-      <c r="D33" s="53" t="n"/>
+      <c r="B33" s="42" t="n"/>
+      <c r="C33" s="42" t="n"/>
+      <c r="D33" s="43" t="n"/>
       <c r="E33" s="53">
         <f>SUM(E5:E32)</f>
         <v/>
@@ -26032,6 +26826,880 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A33:D33"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>T.B.K JH — REKAPITULASI HARIAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="58" t="inlineStr">
+        <is>
+          <t>Data Bal Gudang Induk Tanggal: 3 September 2026 (Kamis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="56" t="inlineStr">
+        <is>
+          <t>No Gud</t>
+        </is>
+      </c>
+      <c r="C4" s="56" t="inlineStr">
+        <is>
+          <t>Nomor Barkot</t>
+        </is>
+      </c>
+      <c r="D4" s="56" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="56" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="56" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="56" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="59" t="n">
+        <v>698</v>
+      </c>
+      <c r="C5" s="60" t="inlineStr">
+        <is>
+          <t>35489</t>
+        </is>
+      </c>
+      <c r="D5" s="59" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E5" s="59" t="n">
+        <v>33</v>
+      </c>
+      <c r="F5" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="59" t="n">
+        <v>699</v>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>35490</t>
+        </is>
+      </c>
+      <c r="D6" s="59" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E6" s="59" t="n">
+        <v>50</v>
+      </c>
+      <c r="F6" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="59" t="n">
+        <v>697</v>
+      </c>
+      <c r="C7" s="60" t="inlineStr">
+        <is>
+          <t>39096</t>
+        </is>
+      </c>
+      <c r="D7" s="59" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E7" s="59" t="n">
+        <v>44</v>
+      </c>
+      <c r="F7" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G7" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="59" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="59" t="n">
+        <v>696</v>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>39097</t>
+        </is>
+      </c>
+      <c r="D8" s="59" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E8" s="59" t="n">
+        <v>39</v>
+      </c>
+      <c r="F8" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="59" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="59" t="n">
+        <v>692</v>
+      </c>
+      <c r="C9" s="60" t="inlineStr">
+        <is>
+          <t>39780</t>
+        </is>
+      </c>
+      <c r="D9" s="59" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E9" s="59" t="n">
+        <v>35</v>
+      </c>
+      <c r="F9" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="59" t="n">
+        <v>693</v>
+      </c>
+      <c r="C10" s="60" t="inlineStr">
+        <is>
+          <t>39098</t>
+        </is>
+      </c>
+      <c r="D10" s="59" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E10" s="59" t="n">
+        <v>37</v>
+      </c>
+      <c r="F10" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="59" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="59" t="n">
+        <v>694</v>
+      </c>
+      <c r="C11" s="60" t="inlineStr">
+        <is>
+          <t>39092</t>
+        </is>
+      </c>
+      <c r="D11" s="59" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E11" s="59" t="n">
+        <v>38</v>
+      </c>
+      <c r="F11" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="59" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="59" t="n">
+        <v>695</v>
+      </c>
+      <c r="C12" s="60" t="inlineStr">
+        <is>
+          <t>39091</t>
+        </is>
+      </c>
+      <c r="D12" s="59" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E12" s="59" t="n">
+        <v>43</v>
+      </c>
+      <c r="F12" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="59" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="59" t="n">
+        <v>688</v>
+      </c>
+      <c r="C13" s="60" t="inlineStr">
+        <is>
+          <t>39095</t>
+        </is>
+      </c>
+      <c r="D13" s="59" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E13" s="59" t="n">
+        <v>41</v>
+      </c>
+      <c r="F13" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="59" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="59" t="n">
+        <v>700</v>
+      </c>
+      <c r="C14" s="60" t="inlineStr">
+        <is>
+          <t>39779</t>
+        </is>
+      </c>
+      <c r="D14" s="59" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E14" s="59" t="n">
+        <v>37</v>
+      </c>
+      <c r="F14" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="59" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="59" t="n">
+        <v>691</v>
+      </c>
+      <c r="C15" s="60" t="inlineStr">
+        <is>
+          <t>39778</t>
+        </is>
+      </c>
+      <c r="D15" s="59" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E15" s="59" t="n">
+        <v>35</v>
+      </c>
+      <c r="F15" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="59" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="59" t="n">
+        <v>701</v>
+      </c>
+      <c r="C16" s="60" t="inlineStr">
+        <is>
+          <t>39776</t>
+        </is>
+      </c>
+      <c r="D16" s="59" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E16" s="59" t="n">
+        <v>35</v>
+      </c>
+      <c r="F16" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="59" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="59" t="n">
+        <v>689</v>
+      </c>
+      <c r="C17" s="60" t="inlineStr">
+        <is>
+          <t>39094</t>
+        </is>
+      </c>
+      <c r="D17" s="59" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E17" s="59" t="n">
+        <v>38</v>
+      </c>
+      <c r="F17" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="59" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="59" t="n">
+        <v>702</v>
+      </c>
+      <c r="C18" s="60" t="inlineStr">
+        <is>
+          <t>39093</t>
+        </is>
+      </c>
+      <c r="D18" s="59" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E18" s="59" t="n">
+        <v>50</v>
+      </c>
+      <c r="F18" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="59" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="59" t="n">
+        <v>690</v>
+      </c>
+      <c r="C19" s="60" t="inlineStr">
+        <is>
+          <t>39777</t>
+        </is>
+      </c>
+      <c r="D19" s="59" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E19" s="59" t="n">
+        <v>35</v>
+      </c>
+      <c r="F19" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="59" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="59" t="n">
+        <v>703</v>
+      </c>
+      <c r="C20" s="60" t="inlineStr">
+        <is>
+          <t>39089</t>
+        </is>
+      </c>
+      <c r="D20" s="59" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E20" s="59" t="n">
+        <v>45</v>
+      </c>
+      <c r="F20" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="59" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="59" t="n">
+        <v>687</v>
+      </c>
+      <c r="C21" s="60" t="inlineStr">
+        <is>
+          <t>39090</t>
+        </is>
+      </c>
+      <c r="D21" s="59" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E21" s="59" t="n">
+        <v>41</v>
+      </c>
+      <c r="F21" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="59" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="59" t="n">
+        <v>704</v>
+      </c>
+      <c r="C22" s="60" t="inlineStr">
+        <is>
+          <t>39088</t>
+        </is>
+      </c>
+      <c r="D22" s="59" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E22" s="59" t="n">
+        <v>32</v>
+      </c>
+      <c r="F22" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="59" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="59" t="n">
+        <v>705</v>
+      </c>
+      <c r="C23" s="60" t="inlineStr">
+        <is>
+          <t>39775</t>
+        </is>
+      </c>
+      <c r="D23" s="59" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E23" s="59" t="n">
+        <v>34</v>
+      </c>
+      <c r="F23" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="59" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="59" t="n">
+        <v>706</v>
+      </c>
+      <c r="C24" s="60" t="inlineStr">
+        <is>
+          <t>39774</t>
+        </is>
+      </c>
+      <c r="D24" s="59" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E24" s="59" t="n">
+        <v>40</v>
+      </c>
+      <c r="F24" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="59" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="59" t="n">
+        <v>707</v>
+      </c>
+      <c r="C25" s="60" t="inlineStr">
+        <is>
+          <t>39086</t>
+        </is>
+      </c>
+      <c r="D25" s="59" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E25" s="59" t="n">
+        <v>48</v>
+      </c>
+      <c r="F25" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G25" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="59" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="59" t="n">
+        <v>708</v>
+      </c>
+      <c r="C26" s="60" t="inlineStr">
+        <is>
+          <t>39084</t>
+        </is>
+      </c>
+      <c r="D26" s="59" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E26" s="59" t="n">
+        <v>35</v>
+      </c>
+      <c r="F26" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G26" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="59" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="59" t="n">
+        <v>709</v>
+      </c>
+      <c r="C27" s="60" t="inlineStr">
+        <is>
+          <t>39085</t>
+        </is>
+      </c>
+      <c r="D27" s="59" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E27" s="59" t="n">
+        <v>39</v>
+      </c>
+      <c r="F27" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G27" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="59" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="59" t="n">
+        <v>710</v>
+      </c>
+      <c r="C28" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D28" s="59" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E28" s="59" t="n">
+        <v>31</v>
+      </c>
+      <c r="F28" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G28" s="61" t="inlineStr">
+        <is>
+          <t>@60.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="59" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="59" t="n">
+        <v>711</v>
+      </c>
+      <c r="C29" s="60" t="inlineStr">
+        <is>
+          <t>39087</t>
+        </is>
+      </c>
+      <c r="D29" s="59" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E29" s="59" t="n">
+        <v>38</v>
+      </c>
+      <c r="F29" s="59" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G29" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="56" t="inlineStr">
+        <is>
+          <t>TOTAL (25 BAL)</t>
+        </is>
+      </c>
+      <c r="B30" s="56" t="n"/>
+      <c r="C30" s="56" t="n"/>
+      <c r="D30" s="56" t="n"/>
+      <c r="E30" s="56">
+        <f>SUM(E5:E29)</f>
+        <v/>
+      </c>
+      <c r="F30" s="56" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G30" s="56" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A30:D30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update & sync data 4 September 2026 (32 bal), rekap master buku grade induk, bump cache version v4.3
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -22,6 +22,7 @@
     <sheet name="1 September" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="2 September" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="3 September" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="4 September" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,7 +34,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;kg&quot;"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -173,6 +174,20 @@
       <name val="Segoe UI"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -236,7 +251,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -408,11 +423,69 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -582,6 +655,30 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -948,7 +1045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H576"/>
+  <dimension ref="A1:H608"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -971,7 +1068,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Laporan Lengkap No Gudang, Nomor Barcode, Grade, dan Berat (Kg) Semua Tanggal (21 Agustus - 3 September 2026)</t>
+          <t>Laporan Lengkap No Gudang, Nomor Barcode, Grade, dan Berat (Kg) Semua Tanggal (21 Agustus - 4 September 2026)</t>
         </is>
       </c>
     </row>
@@ -21323,33 +21420,1186 @@
         </is>
       </c>
     </row>
-    <row r="576" ht="22" customHeight="1">
-      <c r="A576" s="56" t="inlineStr">
-        <is>
-          <t>TOTAL KESELURUHAN (571 BAL)</t>
-        </is>
-      </c>
-      <c r="B576" s="56" t="n"/>
-      <c r="C576" s="56" t="n"/>
-      <c r="D576" s="56" t="n"/>
-      <c r="E576" s="56" t="n"/>
-      <c r="F576" s="56">
-        <f>SUM(F5:F575)</f>
+    <row r="576" ht="20" customHeight="1">
+      <c r="A576" s="62" t="n">
+        <v>572</v>
+      </c>
+      <c r="B576" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C576" s="63" t="n">
+        <v>712</v>
+      </c>
+      <c r="D576" s="64" t="inlineStr">
+        <is>
+          <t>39604</t>
+        </is>
+      </c>
+      <c r="E576" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F576" s="62" t="n">
+        <v>44</v>
+      </c>
+      <c r="G576" s="62" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H576" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="577" ht="20" customHeight="1">
+      <c r="A577" s="63" t="n">
+        <v>573</v>
+      </c>
+      <c r="B577" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C577" s="63" t="n">
+        <v>713</v>
+      </c>
+      <c r="D577" s="64" t="inlineStr">
+        <is>
+          <t>39603</t>
+        </is>
+      </c>
+      <c r="E577" s="63" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F577" s="63" t="n">
+        <v>48</v>
+      </c>
+      <c r="G577" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H577" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="578" ht="20" customHeight="1">
+      <c r="A578" s="63" t="n">
+        <v>574</v>
+      </c>
+      <c r="B578" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C578" s="63" t="n">
+        <v>714</v>
+      </c>
+      <c r="D578" s="64" t="inlineStr">
+        <is>
+          <t>39605</t>
+        </is>
+      </c>
+      <c r="E578" s="63" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F578" s="63" t="n">
+        <v>44</v>
+      </c>
+      <c r="G578" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H578" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="579" ht="20" customHeight="1">
+      <c r="A579" s="63" t="n">
+        <v>575</v>
+      </c>
+      <c r="B579" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C579" s="63" t="n">
+        <v>716</v>
+      </c>
+      <c r="D579" s="64" t="inlineStr">
+        <is>
+          <t>39608</t>
+        </is>
+      </c>
+      <c r="E579" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F579" s="63" t="n">
+        <v>43</v>
+      </c>
+      <c r="G579" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H579" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="580" ht="20" customHeight="1">
+      <c r="A580" s="63" t="n">
+        <v>576</v>
+      </c>
+      <c r="B580" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C580" s="63" t="n">
+        <v>717</v>
+      </c>
+      <c r="D580" s="64" t="inlineStr">
+        <is>
+          <t>39610</t>
+        </is>
+      </c>
+      <c r="E580" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F580" s="63" t="n">
+        <v>42</v>
+      </c>
+      <c r="G580" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H580" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="581" ht="20" customHeight="1">
+      <c r="A581" s="63" t="n">
+        <v>577</v>
+      </c>
+      <c r="B581" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C581" s="63" t="n">
+        <v>718</v>
+      </c>
+      <c r="D581" s="64" t="inlineStr">
+        <is>
+          <t>39607</t>
+        </is>
+      </c>
+      <c r="E581" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F581" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="G581" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H581" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="582" ht="20" customHeight="1">
+      <c r="A582" s="63" t="n">
+        <v>578</v>
+      </c>
+      <c r="B582" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C582" s="63" t="n">
+        <v>720</v>
+      </c>
+      <c r="D582" s="64" t="inlineStr">
+        <is>
+          <t>39557</t>
+        </is>
+      </c>
+      <c r="E582" s="63" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F582" s="63" t="n">
+        <v>37</v>
+      </c>
+      <c r="G582" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H582" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="583" ht="20" customHeight="1">
+      <c r="A583" s="63" t="n">
+        <v>579</v>
+      </c>
+      <c r="B583" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C583" s="63" t="n">
+        <v>721</v>
+      </c>
+      <c r="D583" s="64" t="inlineStr">
+        <is>
+          <t>39606</t>
+        </is>
+      </c>
+      <c r="E583" s="63" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F583" s="63" t="n">
+        <v>40</v>
+      </c>
+      <c r="G583" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H583" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="584" ht="20" customHeight="1">
+      <c r="A584" s="63" t="n">
+        <v>580</v>
+      </c>
+      <c r="B584" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C584" s="63" t="n">
+        <v>722</v>
+      </c>
+      <c r="D584" s="64" t="inlineStr">
+        <is>
+          <t>39609</t>
+        </is>
+      </c>
+      <c r="E584" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F584" s="63" t="n">
+        <v>43</v>
+      </c>
+      <c r="G584" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H584" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="585" ht="20" customHeight="1">
+      <c r="A585" s="63" t="n">
+        <v>581</v>
+      </c>
+      <c r="B585" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C585" s="63" t="n">
+        <v>723</v>
+      </c>
+      <c r="D585" s="64" t="inlineStr">
+        <is>
+          <t>39559</t>
+        </is>
+      </c>
+      <c r="E585" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F585" s="63" t="n">
+        <v>39</v>
+      </c>
+      <c r="G585" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H585" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="586" ht="20" customHeight="1">
+      <c r="A586" s="63" t="n">
+        <v>582</v>
+      </c>
+      <c r="B586" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C586" s="63" t="n">
+        <v>724</v>
+      </c>
+      <c r="D586" s="64" t="inlineStr">
+        <is>
+          <t>39554</t>
+        </is>
+      </c>
+      <c r="E586" s="63" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F586" s="63" t="n">
+        <v>42</v>
+      </c>
+      <c r="G586" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H586" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="587" ht="20" customHeight="1">
+      <c r="A587" s="63" t="n">
+        <v>583</v>
+      </c>
+      <c r="B587" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C587" s="63" t="n">
+        <v>725</v>
+      </c>
+      <c r="D587" s="64" t="inlineStr">
+        <is>
+          <t>39558</t>
+        </is>
+      </c>
+      <c r="E587" s="63" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="F587" s="63" t="n">
+        <v>36</v>
+      </c>
+      <c r="G587" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H587" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="588" ht="20" customHeight="1">
+      <c r="A588" s="63" t="n">
+        <v>584</v>
+      </c>
+      <c r="B588" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C588" s="63" t="n">
+        <v>726</v>
+      </c>
+      <c r="D588" s="64" t="inlineStr">
+        <is>
+          <t>39555</t>
+        </is>
+      </c>
+      <c r="E588" s="63" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F588" s="63" t="n">
+        <v>40</v>
+      </c>
+      <c r="G588" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H588" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="589" ht="20" customHeight="1">
+      <c r="A589" s="63" t="n">
+        <v>585</v>
+      </c>
+      <c r="B589" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C589" s="63" t="n">
+        <v>727</v>
+      </c>
+      <c r="D589" s="64" t="inlineStr">
+        <is>
+          <t>39556</t>
+        </is>
+      </c>
+      <c r="E589" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F589" s="63" t="n">
+        <v>45</v>
+      </c>
+      <c r="G589" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H589" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="590" ht="20" customHeight="1">
+      <c r="A590" s="63" t="n">
+        <v>586</v>
+      </c>
+      <c r="B590" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C590" s="63" t="n">
+        <v>728</v>
+      </c>
+      <c r="D590" s="64" t="inlineStr">
+        <is>
+          <t>39440</t>
+        </is>
+      </c>
+      <c r="E590" s="63" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F590" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="G590" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H590" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="591" ht="20" customHeight="1">
+      <c r="A591" s="63" t="n">
+        <v>587</v>
+      </c>
+      <c r="B591" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C591" s="63" t="n">
+        <v>729</v>
+      </c>
+      <c r="D591" s="64" t="inlineStr">
+        <is>
+          <t>39439</t>
+        </is>
+      </c>
+      <c r="E591" s="63" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F591" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="G591" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H591" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="592" ht="20" customHeight="1">
+      <c r="A592" s="63" t="n">
+        <v>588</v>
+      </c>
+      <c r="B592" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C592" s="63" t="n">
+        <v>730</v>
+      </c>
+      <c r="D592" s="64" t="inlineStr">
+        <is>
+          <t>39441</t>
+        </is>
+      </c>
+      <c r="E592" s="63" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F592" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="G592" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H592" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="593" ht="20" customHeight="1">
+      <c r="A593" s="63" t="n">
+        <v>589</v>
+      </c>
+      <c r="B593" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C593" s="63" t="n">
+        <v>731</v>
+      </c>
+      <c r="D593" s="64" t="inlineStr">
+        <is>
+          <t>39553</t>
+        </is>
+      </c>
+      <c r="E593" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F593" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="G593" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H593" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="594" ht="20" customHeight="1">
+      <c r="A594" s="63" t="n">
+        <v>590</v>
+      </c>
+      <c r="B594" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C594" s="63" t="n">
+        <v>732</v>
+      </c>
+      <c r="D594" s="64" t="inlineStr">
+        <is>
+          <t>39550</t>
+        </is>
+      </c>
+      <c r="E594" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F594" s="63" t="n">
+        <v>30</v>
+      </c>
+      <c r="G594" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H594" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="595" ht="20" customHeight="1">
+      <c r="A595" s="63" t="n">
+        <v>591</v>
+      </c>
+      <c r="B595" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C595" s="63" t="n">
+        <v>733</v>
+      </c>
+      <c r="D595" s="64" t="inlineStr">
+        <is>
+          <t>39552</t>
+        </is>
+      </c>
+      <c r="E595" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F595" s="63" t="n">
+        <v>33</v>
+      </c>
+      <c r="G595" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H595" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="596" ht="20" customHeight="1">
+      <c r="A596" s="63" t="n">
+        <v>592</v>
+      </c>
+      <c r="B596" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C596" s="63" t="n">
+        <v>734</v>
+      </c>
+      <c r="D596" s="64" t="inlineStr">
+        <is>
+          <t>39551</t>
+        </is>
+      </c>
+      <c r="E596" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F596" s="63" t="n">
+        <v>35</v>
+      </c>
+      <c r="G596" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H596" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="597" ht="20" customHeight="1">
+      <c r="A597" s="63" t="n">
+        <v>593</v>
+      </c>
+      <c r="B597" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C597" s="63" t="n">
+        <v>735</v>
+      </c>
+      <c r="D597" s="64" t="inlineStr">
+        <is>
+          <t>39549</t>
+        </is>
+      </c>
+      <c r="E597" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F597" s="63" t="n">
+        <v>35</v>
+      </c>
+      <c r="G597" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H597" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="598" ht="20" customHeight="1">
+      <c r="A598" s="63" t="n">
+        <v>594</v>
+      </c>
+      <c r="B598" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C598" s="63" t="n">
+        <v>737</v>
+      </c>
+      <c r="D598" s="64" t="inlineStr">
+        <is>
+          <t>39167</t>
+        </is>
+      </c>
+      <c r="E598" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F598" s="63" t="n">
+        <v>35</v>
+      </c>
+      <c r="G598" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H598" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="599" ht="20" customHeight="1">
+      <c r="A599" s="63" t="n">
+        <v>595</v>
+      </c>
+      <c r="B599" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C599" s="63" t="n">
+        <v>738</v>
+      </c>
+      <c r="D599" s="64" t="inlineStr">
+        <is>
+          <t>39166</t>
+        </is>
+      </c>
+      <c r="E599" s="63" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F599" s="63" t="n">
+        <v>32</v>
+      </c>
+      <c r="G599" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H599" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="600" ht="20" customHeight="1">
+      <c r="A600" s="63" t="n">
+        <v>596</v>
+      </c>
+      <c r="B600" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C600" s="63" t="n">
+        <v>739</v>
+      </c>
+      <c r="D600" s="64" t="inlineStr">
+        <is>
+          <t>39165</t>
+        </is>
+      </c>
+      <c r="E600" s="63" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F600" s="63" t="n">
+        <v>31</v>
+      </c>
+      <c r="G600" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H600" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="601" ht="20" customHeight="1">
+      <c r="A601" s="63" t="n">
+        <v>597</v>
+      </c>
+      <c r="B601" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C601" s="63" t="n">
+        <v>741</v>
+      </c>
+      <c r="D601" s="64" t="inlineStr">
+        <is>
+          <t>39560</t>
+        </is>
+      </c>
+      <c r="E601" s="63" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F601" s="63" t="n">
+        <v>35</v>
+      </c>
+      <c r="G601" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H601" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="602" ht="20" customHeight="1">
+      <c r="A602" s="63" t="n">
+        <v>598</v>
+      </c>
+      <c r="B602" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C602" s="63" t="n">
+        <v>743</v>
+      </c>
+      <c r="D602" s="64" t="inlineStr">
+        <is>
+          <t>39164</t>
+        </is>
+      </c>
+      <c r="E602" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F602" s="63" t="n">
+        <v>34</v>
+      </c>
+      <c r="G602" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H602" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="603" ht="20" customHeight="1">
+      <c r="A603" s="63" t="n">
+        <v>599</v>
+      </c>
+      <c r="B603" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C603" s="63" t="n">
+        <v>715</v>
+      </c>
+      <c r="D603" s="64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E603" s="63" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F603" s="63" t="n">
+        <v>46</v>
+      </c>
+      <c r="G603" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H603" s="65" t="inlineStr">
+        <is>
+          <t>67 ngoro</t>
+        </is>
+      </c>
+    </row>
+    <row r="604" ht="20" customHeight="1">
+      <c r="A604" s="63" t="n">
+        <v>600</v>
+      </c>
+      <c r="B604" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C604" s="63" t="n">
+        <v>719</v>
+      </c>
+      <c r="D604" s="64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E604" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F604" s="63" t="n">
+        <v>45</v>
+      </c>
+      <c r="G604" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="H604" s="65" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+    </row>
+    <row r="605" ht="20" customHeight="1">
+      <c r="A605" s="63" t="n">
+        <v>601</v>
+      </c>
+      <c r="B605" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C605" s="63" t="n">
+        <v>736</v>
+      </c>
+      <c r="D605" s="64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E605" s="63" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="F605" s="63" t="n">
+        <v>39</v>
+      </c>
+      <c r="G605" s="63" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="H605" s="65" t="inlineStr">
+        <is>
+          <t>out ggal tapelan</t>
+        </is>
+      </c>
+    </row>
+    <row r="606" ht="20" customHeight="1">
+      <c r="A606" s="63" t="n">
+        <v>602</v>
+      </c>
+      <c r="B606" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C606" s="63" t="n">
+        <v>740</v>
+      </c>
+      <c r="D606" s="64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E606" s="63" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F606" s="63" t="n">
+        <v>45</v>
+      </c>
+      <c r="G606" s="63" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="H606" s="65" t="inlineStr">
+        <is>
+          <t>out ggal tapelan</t>
+        </is>
+      </c>
+    </row>
+    <row r="607" ht="20" customHeight="1">
+      <c r="A607" s="63" t="n">
+        <v>603</v>
+      </c>
+      <c r="B607" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C607" s="63" t="n">
+        <v>742</v>
+      </c>
+      <c r="D607" s="64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E607" s="63" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F607" s="63" t="n">
+        <v>36</v>
+      </c>
+      <c r="G607" s="63" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="H607" s="65" t="inlineStr">
+        <is>
+          <t>mote</t>
+        </is>
+      </c>
+    </row>
+    <row r="608" ht="24" customHeight="1">
+      <c r="A608" s="66" t="inlineStr">
+        <is>
+          <t>TOTAL KESELURUHAN (603 BAL)</t>
+        </is>
+      </c>
+      <c r="B608" s="67" t="n"/>
+      <c r="C608" s="67" t="n"/>
+      <c r="D608" s="67" t="n"/>
+      <c r="E608" s="67" t="n"/>
+      <c r="F608" s="66">
+        <f>SUM(F5:F607)</f>
         <v/>
       </c>
-      <c r="G576" s="56" t="inlineStr">
+      <c r="G608" s="66" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
       </c>
+      <c r="H608" s="67" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A608:E608"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A463:E463"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A523:E523"/>
-    <mergeCell ref="A576:E576"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27681,9 +28931,9 @@
           <t>TOTAL (25 BAL)</t>
         </is>
       </c>
-      <c r="B30" s="56" t="n"/>
-      <c r="C30" s="56" t="n"/>
-      <c r="D30" s="56" t="n"/>
+      <c r="B30" s="68" t="n"/>
+      <c r="C30" s="68" t="n"/>
+      <c r="D30" s="69" t="n"/>
       <c r="E30" s="56">
         <f>SUM(E5:E29)</f>
         <v/>
@@ -27700,6 +28950,1097 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A30:D30"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="70" t="inlineStr">
+        <is>
+          <t>T.B.K JH — REKAPITULASI HARIAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="71" t="inlineStr">
+        <is>
+          <t>Data Bal Gudang Induk Tanggal: 4 September 2026 (Jumat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="66" t="inlineStr">
+        <is>
+          <t>No Gud</t>
+        </is>
+      </c>
+      <c r="C4" s="66" t="inlineStr">
+        <is>
+          <t>Nomor Barkot</t>
+        </is>
+      </c>
+      <c r="D4" s="66" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="66" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="66" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="66" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="63" t="n">
+        <v>712</v>
+      </c>
+      <c r="C5" s="64" t="inlineStr">
+        <is>
+          <t>39604</t>
+        </is>
+      </c>
+      <c r="D5" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E5" s="63" t="n">
+        <v>44</v>
+      </c>
+      <c r="F5" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="63" t="n">
+        <v>713</v>
+      </c>
+      <c r="C6" s="64" t="inlineStr">
+        <is>
+          <t>39603</t>
+        </is>
+      </c>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E6" s="63" t="n">
+        <v>48</v>
+      </c>
+      <c r="F6" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="63" t="n">
+        <v>714</v>
+      </c>
+      <c r="C7" s="64" t="inlineStr">
+        <is>
+          <t>39605</t>
+        </is>
+      </c>
+      <c r="D7" s="63" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E7" s="63" t="n">
+        <v>44</v>
+      </c>
+      <c r="F7" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G7" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="63" t="n">
+        <v>716</v>
+      </c>
+      <c r="C8" s="64" t="inlineStr">
+        <is>
+          <t>39608</t>
+        </is>
+      </c>
+      <c r="D8" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E8" s="63" t="n">
+        <v>43</v>
+      </c>
+      <c r="F8" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="63" t="n">
+        <v>717</v>
+      </c>
+      <c r="C9" s="64" t="inlineStr">
+        <is>
+          <t>39610</t>
+        </is>
+      </c>
+      <c r="D9" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E9" s="63" t="n">
+        <v>42</v>
+      </c>
+      <c r="F9" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="63" t="n">
+        <v>718</v>
+      </c>
+      <c r="C10" s="64" t="inlineStr">
+        <is>
+          <t>39607</t>
+        </is>
+      </c>
+      <c r="D10" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E10" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="F10" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="63" t="n">
+        <v>720</v>
+      </c>
+      <c r="C11" s="64" t="inlineStr">
+        <is>
+          <t>39557</t>
+        </is>
+      </c>
+      <c r="D11" s="63" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E11" s="63" t="n">
+        <v>37</v>
+      </c>
+      <c r="F11" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="63" t="n">
+        <v>721</v>
+      </c>
+      <c r="C12" s="64" t="inlineStr">
+        <is>
+          <t>39606</t>
+        </is>
+      </c>
+      <c r="D12" s="63" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E12" s="63" t="n">
+        <v>40</v>
+      </c>
+      <c r="F12" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="63" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="63" t="n">
+        <v>722</v>
+      </c>
+      <c r="C13" s="64" t="inlineStr">
+        <is>
+          <t>39609</t>
+        </is>
+      </c>
+      <c r="D13" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E13" s="63" t="n">
+        <v>43</v>
+      </c>
+      <c r="F13" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="63" t="n">
+        <v>723</v>
+      </c>
+      <c r="C14" s="64" t="inlineStr">
+        <is>
+          <t>39559</t>
+        </is>
+      </c>
+      <c r="D14" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E14" s="63" t="n">
+        <v>39</v>
+      </c>
+      <c r="F14" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="63" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="63" t="n">
+        <v>724</v>
+      </c>
+      <c r="C15" s="64" t="inlineStr">
+        <is>
+          <t>39554</t>
+        </is>
+      </c>
+      <c r="D15" s="63" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E15" s="63" t="n">
+        <v>42</v>
+      </c>
+      <c r="F15" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="63" t="n">
+        <v>725</v>
+      </c>
+      <c r="C16" s="64" t="inlineStr">
+        <is>
+          <t>39558</t>
+        </is>
+      </c>
+      <c r="D16" s="63" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="E16" s="63" t="n">
+        <v>36</v>
+      </c>
+      <c r="F16" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="63" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="63" t="n">
+        <v>726</v>
+      </c>
+      <c r="C17" s="64" t="inlineStr">
+        <is>
+          <t>39555</t>
+        </is>
+      </c>
+      <c r="D17" s="63" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E17" s="63" t="n">
+        <v>40</v>
+      </c>
+      <c r="F17" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="63" t="n">
+        <v>727</v>
+      </c>
+      <c r="C18" s="64" t="inlineStr">
+        <is>
+          <t>39556</t>
+        </is>
+      </c>
+      <c r="D18" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E18" s="63" t="n">
+        <v>45</v>
+      </c>
+      <c r="F18" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="63" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="63" t="n">
+        <v>728</v>
+      </c>
+      <c r="C19" s="64" t="inlineStr">
+        <is>
+          <t>39440</t>
+        </is>
+      </c>
+      <c r="D19" s="63" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E19" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="F19" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="63" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="63" t="n">
+        <v>729</v>
+      </c>
+      <c r="C20" s="64" t="inlineStr">
+        <is>
+          <t>39439</t>
+        </is>
+      </c>
+      <c r="D20" s="63" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E20" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="F20" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="63" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="63" t="n">
+        <v>730</v>
+      </c>
+      <c r="C21" s="64" t="inlineStr">
+        <is>
+          <t>39441</t>
+        </is>
+      </c>
+      <c r="D21" s="63" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E21" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="F21" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="63" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="63" t="n">
+        <v>731</v>
+      </c>
+      <c r="C22" s="64" t="inlineStr">
+        <is>
+          <t>39553</t>
+        </is>
+      </c>
+      <c r="D22" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E22" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="F22" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="63" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="63" t="n">
+        <v>732</v>
+      </c>
+      <c r="C23" s="64" t="inlineStr">
+        <is>
+          <t>39550</t>
+        </is>
+      </c>
+      <c r="D23" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E23" s="63" t="n">
+        <v>30</v>
+      </c>
+      <c r="F23" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="63" t="n">
+        <v>733</v>
+      </c>
+      <c r="C24" s="64" t="inlineStr">
+        <is>
+          <t>39552</t>
+        </is>
+      </c>
+      <c r="D24" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E24" s="63" t="n">
+        <v>33</v>
+      </c>
+      <c r="F24" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="63" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="63" t="n">
+        <v>734</v>
+      </c>
+      <c r="C25" s="64" t="inlineStr">
+        <is>
+          <t>39551</t>
+        </is>
+      </c>
+      <c r="D25" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E25" s="63" t="n">
+        <v>35</v>
+      </c>
+      <c r="F25" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G25" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="63" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="63" t="n">
+        <v>735</v>
+      </c>
+      <c r="C26" s="64" t="inlineStr">
+        <is>
+          <t>39549</t>
+        </is>
+      </c>
+      <c r="D26" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E26" s="63" t="n">
+        <v>35</v>
+      </c>
+      <c r="F26" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G26" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="63" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="63" t="n">
+        <v>737</v>
+      </c>
+      <c r="C27" s="64" t="inlineStr">
+        <is>
+          <t>39167</t>
+        </is>
+      </c>
+      <c r="D27" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E27" s="63" t="n">
+        <v>35</v>
+      </c>
+      <c r="F27" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G27" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="63" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="63" t="n">
+        <v>738</v>
+      </c>
+      <c r="C28" s="64" t="inlineStr">
+        <is>
+          <t>39166</t>
+        </is>
+      </c>
+      <c r="D28" s="63" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E28" s="63" t="n">
+        <v>32</v>
+      </c>
+      <c r="F28" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G28" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="63" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="63" t="n">
+        <v>739</v>
+      </c>
+      <c r="C29" s="64" t="inlineStr">
+        <is>
+          <t>39165</t>
+        </is>
+      </c>
+      <c r="D29" s="63" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E29" s="63" t="n">
+        <v>31</v>
+      </c>
+      <c r="F29" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G29" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="63" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="63" t="n">
+        <v>741</v>
+      </c>
+      <c r="C30" s="64" t="inlineStr">
+        <is>
+          <t>39560</t>
+        </is>
+      </c>
+      <c r="D30" s="63" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E30" s="63" t="n">
+        <v>35</v>
+      </c>
+      <c r="F30" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G30" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="63" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="63" t="n">
+        <v>743</v>
+      </c>
+      <c r="C31" s="64" t="inlineStr">
+        <is>
+          <t>39164</t>
+        </is>
+      </c>
+      <c r="D31" s="63" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E31" s="63" t="n">
+        <v>34</v>
+      </c>
+      <c r="F31" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G31" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="63" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="63" t="n">
+        <v>715</v>
+      </c>
+      <c r="C32" s="64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" s="63" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E32" s="63" t="n">
+        <v>46</v>
+      </c>
+      <c r="F32" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G32" s="65" t="inlineStr">
+        <is>
+          <t>67 ngoro</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="63" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="63" t="n">
+        <v>719</v>
+      </c>
+      <c r="C33" s="64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D33" s="63" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E33" s="63" t="n">
+        <v>45</v>
+      </c>
+      <c r="F33" s="63" t="inlineStr">
+        <is>
+          <t>BELUM SELESAI</t>
+        </is>
+      </c>
+      <c r="G33" s="65" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="63" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="63" t="n">
+        <v>736</v>
+      </c>
+      <c r="C34" s="64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D34" s="63" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="E34" s="63" t="n">
+        <v>39</v>
+      </c>
+      <c r="F34" s="63" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G34" s="65" t="inlineStr">
+        <is>
+          <t>out ggal tapelan</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="63" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="63" t="n">
+        <v>740</v>
+      </c>
+      <c r="C35" s="64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" s="63" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E35" s="63" t="n">
+        <v>45</v>
+      </c>
+      <c r="F35" s="63" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G35" s="65" t="inlineStr">
+        <is>
+          <t>out ggal tapelan</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="63" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="63" t="n">
+        <v>742</v>
+      </c>
+      <c r="C36" s="64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D36" s="63" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E36" s="63" t="n">
+        <v>36</v>
+      </c>
+      <c r="F36" s="63" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G36" s="65" t="inlineStr">
+        <is>
+          <t>mote</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="66" t="inlineStr">
+        <is>
+          <t>TOTAL (32 BAL)</t>
+        </is>
+      </c>
+      <c r="B37" s="67" t="n"/>
+      <c r="C37" s="67" t="n"/>
+      <c r="D37" s="67" t="n"/>
+      <c r="E37" s="66">
+        <f>SUM(E5:E36)</f>
+        <v/>
+      </c>
+      <c r="F37" s="66" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G37" s="67" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>